<commit_message>
feat(mobile): improve mobile layout & box sizing, solid white text on red buttons, update header title, footer developed by WHS
</commit_message>
<xml_diff>
--- a/templates/LJK.xlsx
+++ b/templates/LJK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahyu/research/math-center/upload-apps/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00930A0-CEC5-4046-9957-63304508585C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC8776E-F989-E945-8F71-6612A8F3BCF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{CF4DB2AD-E87A-8A4F-945F-369D44C0138B}"/>
   </bookViews>
@@ -811,122 +811,81 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>1. Gunakan </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>pensil 2B</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t> saja. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>1. Gunakan pensil 2B. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>2. Jaga lembar jawaban agar </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>bersih, kering, dan tidak terlipat</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>2. Pastikan lembar jawaban agar bersih, kering, dan tidak terlipat. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>3. Silang </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>satu pilihan jawaban</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t> dengan penuh dan jelas. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>3. Silang satu pilihan jawaban dengan jelas. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>4. Tuliskan </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>Nama Lengkap dan NPM</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>, lalu silang kotak yang sesuai. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>4. Tuliskan Nama Lengkap dan NIM.</a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>5. Silang </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>5. Isi</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>kotak Fakultas</a:t>
+            <a:rPr lang="en-ID" sz="900" b="0" baseline="0"/>
+            <a:t> f</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t> sesuai fakultas Anda. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>akultas saudara/i dan</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-ID" sz="900" b="0" baseline="0"/>
+            <a:t> k</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>ode soal yang diberikan pengawas. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>6. Tuliskan </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>tanggal ujian</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t> dan bubuhkan tanda tangan pada tempat yang disediakan. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>6. Tuliskan tanggal ujian dan bubuhkan tanda tangan pada tempat yang disediakan. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>7. Jika salah silang, </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>hapus sebersih mungkin</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900"/>
-            <a:t>, lalu silang jawaban yang benar. </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>7. Jika salah silang, hapus sebersih mungkin, lalu silang jawaban yang benar. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>8. Berdoa sebelum mengerjakan dan kerjakan ujian dengan penuh </a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>8. Berdoa sebelum mengerjakan dan kerjakan dengan jujur serta penuh integritas.</a:t>
+            <a:t>integritas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>.</a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>9. Kumpulkan </a:t>
+            <a:rPr lang="en-ID" sz="900" b="0"/>
+            <a:t>9. Kumpulkan LJK kepada pengawas saat ujian selesai.</a:t>
           </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="0"/>
-            <a:t>LJK kepada pengawas saat ujian selesai</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="900" b="1"/>
-            <a:t>.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-ID" sz="900"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
feat(template): update template json with latest calibrated layout
</commit_message>
<xml_diff>
--- a/templates/LJK.xlsx
+++ b/templates/LJK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahyu/research/math-center/upload-apps/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC8776E-F989-E945-8F71-6612A8F3BCF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E87AB51C-E3EE-2A47-94A2-95D237D4B16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{CF4DB2AD-E87A-8A4F-945F-369D44C0138B}"/>
   </bookViews>
@@ -684,6 +684,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -714,21 +729,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5492,47 +5492,47 @@
       <c r="A4" s="5"/>
       <c r="B4" s="20"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="63" t="s">
+      <c r="D4" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="63"/>
-      <c r="O4" s="63"/>
-      <c r="P4" s="63"/>
-      <c r="Q4" s="63"/>
-      <c r="R4" s="63"/>
-      <c r="S4" s="63"/>
-      <c r="T4" s="63"/>
-      <c r="U4" s="63"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="63"/>
-      <c r="X4" s="63"/>
-      <c r="Y4" s="63"/>
-      <c r="Z4" s="63"/>
-      <c r="AA4" s="63"/>
-      <c r="AB4" s="63"/>
-      <c r="AC4" s="63"/>
-      <c r="AD4" s="63"/>
-      <c r="AE4" s="63"/>
-      <c r="AF4" s="63"/>
-      <c r="AG4" s="63"/>
-      <c r="AH4" s="63"/>
-      <c r="AI4" s="63"/>
-      <c r="AJ4" s="63"/>
-      <c r="AK4" s="63"/>
-      <c r="AL4" s="63"/>
-      <c r="AM4" s="63"/>
-      <c r="AN4" s="63"/>
-      <c r="AO4" s="63"/>
-      <c r="AP4" s="64"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="68"/>
+      <c r="S4" s="68"/>
+      <c r="T4" s="68"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Y4" s="68"/>
+      <c r="Z4" s="68"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
+      <c r="AD4" s="68"/>
+      <c r="AE4" s="68"/>
+      <c r="AF4" s="68"/>
+      <c r="AG4" s="68"/>
+      <c r="AH4" s="68"/>
+      <c r="AI4" s="68"/>
+      <c r="AJ4" s="68"/>
+      <c r="AK4" s="68"/>
+      <c r="AL4" s="68"/>
+      <c r="AM4" s="68"/>
+      <c r="AN4" s="68"/>
+      <c r="AO4" s="68"/>
+      <c r="AP4" s="69"/>
       <c r="AQ4" s="33"/>
       <c r="AR4" s="33"/>
       <c r="AS4" s="5"/>
@@ -5545,45 +5545,45 @@
       <c r="A5" s="5"/>
       <c r="B5" s="20"/>
       <c r="C5" s="5"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="63"/>
-      <c r="L5" s="63"/>
-      <c r="M5" s="63"/>
-      <c r="N5" s="63"/>
-      <c r="O5" s="63"/>
-      <c r="P5" s="63"/>
-      <c r="Q5" s="63"/>
-      <c r="R5" s="63"/>
-      <c r="S5" s="63"/>
-      <c r="T5" s="63"/>
-      <c r="U5" s="63"/>
-      <c r="V5" s="63"/>
-      <c r="W5" s="63"/>
-      <c r="X5" s="63"/>
-      <c r="Y5" s="63"/>
-      <c r="Z5" s="63"/>
-      <c r="AA5" s="63"/>
-      <c r="AB5" s="63"/>
-      <c r="AC5" s="63"/>
-      <c r="AD5" s="63"/>
-      <c r="AE5" s="63"/>
-      <c r="AF5" s="63"/>
-      <c r="AG5" s="63"/>
-      <c r="AH5" s="63"/>
-      <c r="AI5" s="63"/>
-      <c r="AJ5" s="63"/>
-      <c r="AK5" s="63"/>
-      <c r="AL5" s="63"/>
-      <c r="AM5" s="63"/>
-      <c r="AN5" s="63"/>
-      <c r="AO5" s="63"/>
-      <c r="AP5" s="64"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
+      <c r="O5" s="68"/>
+      <c r="P5" s="68"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="68"/>
+      <c r="Y5" s="68"/>
+      <c r="Z5" s="68"/>
+      <c r="AA5" s="68"/>
+      <c r="AB5" s="68"/>
+      <c r="AC5" s="68"/>
+      <c r="AD5" s="68"/>
+      <c r="AE5" s="68"/>
+      <c r="AF5" s="68"/>
+      <c r="AG5" s="68"/>
+      <c r="AH5" s="68"/>
+      <c r="AI5" s="68"/>
+      <c r="AJ5" s="68"/>
+      <c r="AK5" s="68"/>
+      <c r="AL5" s="68"/>
+      <c r="AM5" s="68"/>
+      <c r="AN5" s="68"/>
+      <c r="AO5" s="68"/>
+      <c r="AP5" s="69"/>
       <c r="AQ5" s="33"/>
       <c r="AR5" s="33"/>
       <c r="AS5" s="5"/>
@@ -5596,47 +5596,47 @@
       <c r="A6" s="5"/>
       <c r="B6" s="20"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="63" t="s">
+      <c r="D6" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="63"/>
-      <c r="N6" s="63"/>
-      <c r="O6" s="63"/>
-      <c r="P6" s="63"/>
-      <c r="Q6" s="63"/>
-      <c r="R6" s="63"/>
-      <c r="S6" s="63"/>
-      <c r="T6" s="63"/>
-      <c r="U6" s="63"/>
-      <c r="V6" s="63"/>
-      <c r="W6" s="63"/>
-      <c r="X6" s="63"/>
-      <c r="Y6" s="63"/>
-      <c r="Z6" s="63"/>
-      <c r="AA6" s="63"/>
-      <c r="AB6" s="63"/>
-      <c r="AC6" s="63"/>
-      <c r="AD6" s="63"/>
-      <c r="AE6" s="63"/>
-      <c r="AF6" s="63"/>
-      <c r="AG6" s="63"/>
-      <c r="AH6" s="63"/>
-      <c r="AI6" s="63"/>
-      <c r="AJ6" s="63"/>
-      <c r="AK6" s="63"/>
-      <c r="AL6" s="63"/>
-      <c r="AM6" s="63"/>
-      <c r="AN6" s="63"/>
-      <c r="AO6" s="63"/>
-      <c r="AP6" s="64"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
+      <c r="N6" s="68"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="68"/>
+      <c r="Q6" s="68"/>
+      <c r="R6" s="68"/>
+      <c r="S6" s="68"/>
+      <c r="T6" s="68"/>
+      <c r="U6" s="68"/>
+      <c r="V6" s="68"/>
+      <c r="W6" s="68"/>
+      <c r="X6" s="68"/>
+      <c r="Y6" s="68"/>
+      <c r="Z6" s="68"/>
+      <c r="AA6" s="68"/>
+      <c r="AB6" s="68"/>
+      <c r="AC6" s="68"/>
+      <c r="AD6" s="68"/>
+      <c r="AE6" s="68"/>
+      <c r="AF6" s="68"/>
+      <c r="AG6" s="68"/>
+      <c r="AH6" s="68"/>
+      <c r="AI6" s="68"/>
+      <c r="AJ6" s="68"/>
+      <c r="AK6" s="68"/>
+      <c r="AL6" s="68"/>
+      <c r="AM6" s="68"/>
+      <c r="AN6" s="68"/>
+      <c r="AO6" s="68"/>
+      <c r="AP6" s="69"/>
       <c r="AQ6" s="33"/>
       <c r="AR6" s="33"/>
       <c r="AS6" s="5"/>
@@ -5649,47 +5649,47 @@
       <c r="A7" s="5"/>
       <c r="B7" s="20"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="63" t="s">
+      <c r="D7" s="68" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="63"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="63"/>
-      <c r="M7" s="63"/>
-      <c r="N7" s="63"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="63"/>
-      <c r="Q7" s="63"/>
-      <c r="R7" s="63"/>
-      <c r="S7" s="63"/>
-      <c r="T7" s="63"/>
-      <c r="U7" s="63"/>
-      <c r="V7" s="63"/>
-      <c r="W7" s="63"/>
-      <c r="X7" s="63"/>
-      <c r="Y7" s="63"/>
-      <c r="Z7" s="63"/>
-      <c r="AA7" s="63"/>
-      <c r="AB7" s="63"/>
-      <c r="AC7" s="63"/>
-      <c r="AD7" s="63"/>
-      <c r="AE7" s="63"/>
-      <c r="AF7" s="63"/>
-      <c r="AG7" s="63"/>
-      <c r="AH7" s="63"/>
-      <c r="AI7" s="63"/>
-      <c r="AJ7" s="63"/>
-      <c r="AK7" s="63"/>
-      <c r="AL7" s="63"/>
-      <c r="AM7" s="63"/>
-      <c r="AN7" s="63"/>
-      <c r="AO7" s="63"/>
-      <c r="AP7" s="64"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="68"/>
+      <c r="H7" s="68"/>
+      <c r="I7" s="68"/>
+      <c r="J7" s="68"/>
+      <c r="K7" s="68"/>
+      <c r="L7" s="68"/>
+      <c r="M7" s="68"/>
+      <c r="N7" s="68"/>
+      <c r="O7" s="68"/>
+      <c r="P7" s="68"/>
+      <c r="Q7" s="68"/>
+      <c r="R7" s="68"/>
+      <c r="S7" s="68"/>
+      <c r="T7" s="68"/>
+      <c r="U7" s="68"/>
+      <c r="V7" s="68"/>
+      <c r="W7" s="68"/>
+      <c r="X7" s="68"/>
+      <c r="Y7" s="68"/>
+      <c r="Z7" s="68"/>
+      <c r="AA7" s="68"/>
+      <c r="AB7" s="68"/>
+      <c r="AC7" s="68"/>
+      <c r="AD7" s="68"/>
+      <c r="AE7" s="68"/>
+      <c r="AF7" s="68"/>
+      <c r="AG7" s="68"/>
+      <c r="AH7" s="68"/>
+      <c r="AI7" s="68"/>
+      <c r="AJ7" s="68"/>
+      <c r="AK7" s="68"/>
+      <c r="AL7" s="68"/>
+      <c r="AM7" s="68"/>
+      <c r="AN7" s="68"/>
+      <c r="AO7" s="68"/>
+      <c r="AP7" s="69"/>
       <c r="AQ7" s="33"/>
       <c r="AR7" s="33"/>
       <c r="AS7" s="5"/>
@@ -5702,45 +5702,45 @@
       <c r="A8" s="5"/>
       <c r="B8" s="20"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="56"/>
-      <c r="J8" s="56"/>
-      <c r="K8" s="56"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="56"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="56"/>
-      <c r="P8" s="56"/>
-      <c r="Q8" s="56"/>
-      <c r="R8" s="56"/>
-      <c r="S8" s="56"/>
-      <c r="T8" s="56"/>
-      <c r="U8" s="56"/>
-      <c r="V8" s="56"/>
-      <c r="W8" s="56"/>
-      <c r="X8" s="56"/>
-      <c r="Y8" s="56"/>
-      <c r="Z8" s="56"/>
-      <c r="AA8" s="56"/>
-      <c r="AB8" s="56"/>
-      <c r="AC8" s="56"/>
-      <c r="AD8" s="56"/>
-      <c r="AE8" s="56"/>
-      <c r="AF8" s="56"/>
-      <c r="AG8" s="56"/>
-      <c r="AH8" s="56"/>
-      <c r="AI8" s="56"/>
-      <c r="AJ8" s="56"/>
-      <c r="AK8" s="56"/>
-      <c r="AL8" s="56"/>
-      <c r="AM8" s="56"/>
-      <c r="AN8" s="56"/>
-      <c r="AO8" s="56"/>
-      <c r="AP8" s="57"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="61"/>
+      <c r="K8" s="61"/>
+      <c r="L8" s="61"/>
+      <c r="M8" s="61"/>
+      <c r="N8" s="61"/>
+      <c r="O8" s="61"/>
+      <c r="P8" s="61"/>
+      <c r="Q8" s="61"/>
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
+      <c r="T8" s="61"/>
+      <c r="U8" s="61"/>
+      <c r="V8" s="61"/>
+      <c r="W8" s="61"/>
+      <c r="X8" s="61"/>
+      <c r="Y8" s="61"/>
+      <c r="Z8" s="61"/>
+      <c r="AA8" s="61"/>
+      <c r="AB8" s="61"/>
+      <c r="AC8" s="61"/>
+      <c r="AD8" s="61"/>
+      <c r="AE8" s="61"/>
+      <c r="AF8" s="61"/>
+      <c r="AG8" s="61"/>
+      <c r="AH8" s="61"/>
+      <c r="AI8" s="61"/>
+      <c r="AJ8" s="61"/>
+      <c r="AK8" s="61"/>
+      <c r="AL8" s="61"/>
+      <c r="AM8" s="61"/>
+      <c r="AN8" s="61"/>
+      <c r="AO8" s="61"/>
+      <c r="AP8" s="62"/>
       <c r="AQ8" s="33"/>
       <c r="AR8" s="33"/>
       <c r="AS8" s="5"/>
@@ -5753,45 +5753,45 @@
       <c r="A9" s="5"/>
       <c r="B9" s="20"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="61"/>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="61"/>
-      <c r="N9" s="61"/>
-      <c r="O9" s="61"/>
-      <c r="P9" s="61"/>
-      <c r="Q9" s="61"/>
-      <c r="R9" s="61"/>
-      <c r="S9" s="61"/>
-      <c r="T9" s="61"/>
-      <c r="U9" s="61"/>
-      <c r="V9" s="61"/>
-      <c r="W9" s="61"/>
-      <c r="X9" s="61"/>
-      <c r="Y9" s="61"/>
-      <c r="Z9" s="61"/>
-      <c r="AA9" s="61"/>
-      <c r="AB9" s="61"/>
-      <c r="AC9" s="61"/>
-      <c r="AD9" s="61"/>
-      <c r="AE9" s="61"/>
-      <c r="AF9" s="61"/>
-      <c r="AG9" s="61"/>
-      <c r="AH9" s="61"/>
-      <c r="AI9" s="61"/>
-      <c r="AJ9" s="61"/>
-      <c r="AK9" s="61"/>
-      <c r="AL9" s="61"/>
-      <c r="AM9" s="61"/>
-      <c r="AN9" s="61"/>
-      <c r="AO9" s="61"/>
-      <c r="AP9" s="62"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="66"/>
+      <c r="N9" s="66"/>
+      <c r="O9" s="66"/>
+      <c r="P9" s="66"/>
+      <c r="Q9" s="66"/>
+      <c r="R9" s="66"/>
+      <c r="S9" s="66"/>
+      <c r="T9" s="66"/>
+      <c r="U9" s="66"/>
+      <c r="V9" s="66"/>
+      <c r="W9" s="66"/>
+      <c r="X9" s="66"/>
+      <c r="Y9" s="66"/>
+      <c r="Z9" s="66"/>
+      <c r="AA9" s="66"/>
+      <c r="AB9" s="66"/>
+      <c r="AC9" s="66"/>
+      <c r="AD9" s="66"/>
+      <c r="AE9" s="66"/>
+      <c r="AF9" s="66"/>
+      <c r="AG9" s="66"/>
+      <c r="AH9" s="66"/>
+      <c r="AI9" s="66"/>
+      <c r="AJ9" s="66"/>
+      <c r="AK9" s="66"/>
+      <c r="AL9" s="66"/>
+      <c r="AM9" s="66"/>
+      <c r="AN9" s="66"/>
+      <c r="AO9" s="66"/>
+      <c r="AP9" s="67"/>
       <c r="AQ9" s="33"/>
       <c r="AR9" s="33"/>
       <c r="AS9" s="5"/>
@@ -5804,47 +5804,47 @@
       <c r="A10" s="5"/>
       <c r="B10" s="20"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="56" t="s">
+      <c r="D10" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="56"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56"/>
-      <c r="N10" s="56"/>
-      <c r="O10" s="56"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="56"/>
-      <c r="R10" s="56"/>
-      <c r="S10" s="56"/>
-      <c r="T10" s="56"/>
-      <c r="U10" s="56"/>
-      <c r="V10" s="56"/>
-      <c r="W10" s="56"/>
-      <c r="X10" s="56"/>
-      <c r="Y10" s="56"/>
-      <c r="Z10" s="56"/>
-      <c r="AA10" s="56"/>
-      <c r="AB10" s="56"/>
-      <c r="AC10" s="56"/>
-      <c r="AD10" s="56"/>
-      <c r="AE10" s="56"/>
-      <c r="AF10" s="56"/>
-      <c r="AG10" s="56"/>
-      <c r="AH10" s="56"/>
-      <c r="AI10" s="56"/>
-      <c r="AJ10" s="56"/>
-      <c r="AK10" s="56"/>
-      <c r="AL10" s="56"/>
-      <c r="AM10" s="56"/>
-      <c r="AN10" s="56"/>
-      <c r="AO10" s="56"/>
-      <c r="AP10" s="57"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
+      <c r="K10" s="61"/>
+      <c r="L10" s="61"/>
+      <c r="M10" s="61"/>
+      <c r="N10" s="61"/>
+      <c r="O10" s="61"/>
+      <c r="P10" s="61"/>
+      <c r="Q10" s="61"/>
+      <c r="R10" s="61"/>
+      <c r="S10" s="61"/>
+      <c r="T10" s="61"/>
+      <c r="U10" s="61"/>
+      <c r="V10" s="61"/>
+      <c r="W10" s="61"/>
+      <c r="X10" s="61"/>
+      <c r="Y10" s="61"/>
+      <c r="Z10" s="61"/>
+      <c r="AA10" s="61"/>
+      <c r="AB10" s="61"/>
+      <c r="AC10" s="61"/>
+      <c r="AD10" s="61"/>
+      <c r="AE10" s="61"/>
+      <c r="AF10" s="61"/>
+      <c r="AG10" s="61"/>
+      <c r="AH10" s="61"/>
+      <c r="AI10" s="61"/>
+      <c r="AJ10" s="61"/>
+      <c r="AK10" s="61"/>
+      <c r="AL10" s="61"/>
+      <c r="AM10" s="61"/>
+      <c r="AN10" s="61"/>
+      <c r="AO10" s="61"/>
+      <c r="AP10" s="62"/>
       <c r="AQ10" s="33"/>
       <c r="AR10" s="33"/>
       <c r="AS10" s="5"/>
@@ -6267,93 +6267,93 @@
       <c r="A19" s="5"/>
       <c r="B19" s="20"/>
       <c r="C19" s="5"/>
-      <c r="D19" s="58" t="s">
+      <c r="D19" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="58"/>
-      <c r="I19" s="58"/>
-      <c r="J19" s="58"/>
-      <c r="K19" s="58"/>
-      <c r="L19" s="58"/>
-      <c r="M19" s="58"/>
-      <c r="N19" s="58"/>
-      <c r="O19" s="58"/>
-      <c r="P19" s="58"/>
-      <c r="Q19" s="58"/>
-      <c r="R19" s="58"/>
-      <c r="S19" s="58"/>
-      <c r="T19" s="58"/>
-      <c r="U19" s="58"/>
-      <c r="V19" s="58"/>
-      <c r="W19" s="58"/>
-      <c r="X19" s="58"/>
-      <c r="Y19" s="58"/>
-      <c r="Z19" s="58"/>
-      <c r="AA19" s="58"/>
-      <c r="AB19" s="58"/>
-      <c r="AC19" s="58"/>
-      <c r="AD19" s="58"/>
-      <c r="AE19" s="58"/>
-      <c r="AF19" s="58"/>
-      <c r="AG19" s="58"/>
-      <c r="AH19" s="58"/>
-      <c r="AI19" s="58"/>
-      <c r="AJ19" s="58"/>
-      <c r="AK19" s="58"/>
-      <c r="AL19" s="58"/>
-      <c r="AM19" s="58"/>
-      <c r="AN19" s="58"/>
-      <c r="AO19" s="58"/>
-      <c r="AP19" s="58"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="63"/>
+      <c r="K19" s="63"/>
+      <c r="L19" s="63"/>
+      <c r="M19" s="63"/>
+      <c r="N19" s="63"/>
+      <c r="O19" s="63"/>
+      <c r="P19" s="63"/>
+      <c r="Q19" s="63"/>
+      <c r="R19" s="63"/>
+      <c r="S19" s="63"/>
+      <c r="T19" s="63"/>
+      <c r="U19" s="63"/>
+      <c r="V19" s="63"/>
+      <c r="W19" s="63"/>
+      <c r="X19" s="63"/>
+      <c r="Y19" s="63"/>
+      <c r="Z19" s="63"/>
+      <c r="AA19" s="63"/>
+      <c r="AB19" s="63"/>
+      <c r="AC19" s="63"/>
+      <c r="AD19" s="63"/>
+      <c r="AE19" s="63"/>
+      <c r="AF19" s="63"/>
+      <c r="AG19" s="63"/>
+      <c r="AH19" s="63"/>
+      <c r="AI19" s="63"/>
+      <c r="AJ19" s="63"/>
+      <c r="AK19" s="63"/>
+      <c r="AL19" s="63"/>
+      <c r="AM19" s="63"/>
+      <c r="AN19" s="63"/>
+      <c r="AO19" s="63"/>
+      <c r="AP19" s="63"/>
       <c r="AQ19" s="6"/>
       <c r="AR19" s="33"/>
       <c r="AS19" s="5"/>
-      <c r="AT19" s="58" t="s">
+      <c r="AT19" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="AU19" s="58"/>
-      <c r="AV19" s="58"/>
-      <c r="AW19" s="58"/>
-      <c r="AX19" s="58"/>
-      <c r="AY19" s="58"/>
-      <c r="AZ19" s="58"/>
-      <c r="BA19" s="58"/>
-      <c r="BB19" s="58"/>
-      <c r="BC19" s="58"/>
-      <c r="BD19" s="58"/>
-      <c r="BE19" s="58"/>
-      <c r="BF19" s="58"/>
-      <c r="BG19" s="58"/>
-      <c r="BH19" s="58"/>
-      <c r="BI19" s="58"/>
-      <c r="BJ19" s="58"/>
-      <c r="BK19" s="58"/>
-      <c r="BL19" s="58"/>
-      <c r="BM19" s="58"/>
+      <c r="AU19" s="63"/>
+      <c r="AV19" s="63"/>
+      <c r="AW19" s="63"/>
+      <c r="AX19" s="63"/>
+      <c r="AY19" s="63"/>
+      <c r="AZ19" s="63"/>
+      <c r="BA19" s="63"/>
+      <c r="BB19" s="63"/>
+      <c r="BC19" s="63"/>
+      <c r="BD19" s="63"/>
+      <c r="BE19" s="63"/>
+      <c r="BF19" s="63"/>
+      <c r="BG19" s="63"/>
+      <c r="BH19" s="63"/>
+      <c r="BI19" s="63"/>
+      <c r="BJ19" s="63"/>
+      <c r="BK19" s="63"/>
+      <c r="BL19" s="63"/>
+      <c r="BM19" s="63"/>
       <c r="BN19" s="24"/>
       <c r="BO19" s="29"/>
-      <c r="BP19" s="58" t="s">
+      <c r="BP19" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="BQ19" s="58"/>
-      <c r="BR19" s="58"/>
-      <c r="BS19" s="58"/>
-      <c r="BT19" s="58"/>
-      <c r="BU19" s="58"/>
-      <c r="BV19" s="58"/>
+      <c r="BQ19" s="63"/>
+      <c r="BR19" s="63"/>
+      <c r="BS19" s="63"/>
+      <c r="BT19" s="63"/>
+      <c r="BU19" s="63"/>
+      <c r="BV19" s="63"/>
       <c r="BW19" s="45"/>
       <c r="BX19" s="24"/>
       <c r="BY19" s="51"/>
-      <c r="BZ19" s="65" t="s">
+      <c r="BZ19" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="CA19" s="65"/>
-      <c r="CB19" s="65"/>
-      <c r="CC19" s="65"/>
-      <c r="CD19" s="65"/>
+      <c r="CA19" s="70"/>
+      <c r="CB19" s="70"/>
+      <c r="CC19" s="70"/>
+      <c r="CD19" s="70"/>
       <c r="CE19" s="46"/>
       <c r="CF19" s="18"/>
       <c r="CG19" s="6"/>
@@ -6362,85 +6362,85 @@
       <c r="A20" s="5"/>
       <c r="B20" s="20"/>
       <c r="C20" s="9"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="59"/>
-      <c r="I20" s="59"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="59"/>
-      <c r="L20" s="59"/>
-      <c r="M20" s="59"/>
-      <c r="N20" s="59"/>
-      <c r="O20" s="59"/>
-      <c r="P20" s="59"/>
-      <c r="Q20" s="59"/>
-      <c r="R20" s="59"/>
-      <c r="S20" s="59"/>
-      <c r="T20" s="59"/>
-      <c r="U20" s="59"/>
-      <c r="V20" s="59"/>
-      <c r="W20" s="59"/>
-      <c r="X20" s="59"/>
-      <c r="Y20" s="59"/>
-      <c r="Z20" s="59"/>
-      <c r="AA20" s="59"/>
-      <c r="AB20" s="59"/>
-      <c r="AC20" s="59"/>
-      <c r="AD20" s="59"/>
-      <c r="AE20" s="59"/>
-      <c r="AF20" s="59"/>
-      <c r="AG20" s="59"/>
-      <c r="AH20" s="59"/>
-      <c r="AI20" s="59"/>
-      <c r="AJ20" s="59"/>
-      <c r="AK20" s="59"/>
-      <c r="AL20" s="59"/>
-      <c r="AM20" s="59"/>
-      <c r="AN20" s="59"/>
-      <c r="AO20" s="59"/>
-      <c r="AP20" s="59"/>
+      <c r="D20" s="64"/>
+      <c r="E20" s="64"/>
+      <c r="F20" s="64"/>
+      <c r="G20" s="64"/>
+      <c r="H20" s="64"/>
+      <c r="I20" s="64"/>
+      <c r="J20" s="64"/>
+      <c r="K20" s="64"/>
+      <c r="L20" s="64"/>
+      <c r="M20" s="64"/>
+      <c r="N20" s="64"/>
+      <c r="O20" s="64"/>
+      <c r="P20" s="64"/>
+      <c r="Q20" s="64"/>
+      <c r="R20" s="64"/>
+      <c r="S20" s="64"/>
+      <c r="T20" s="64"/>
+      <c r="U20" s="64"/>
+      <c r="V20" s="64"/>
+      <c r="W20" s="64"/>
+      <c r="X20" s="64"/>
+      <c r="Y20" s="64"/>
+      <c r="Z20" s="64"/>
+      <c r="AA20" s="64"/>
+      <c r="AB20" s="64"/>
+      <c r="AC20" s="64"/>
+      <c r="AD20" s="64"/>
+      <c r="AE20" s="64"/>
+      <c r="AF20" s="64"/>
+      <c r="AG20" s="64"/>
+      <c r="AH20" s="64"/>
+      <c r="AI20" s="64"/>
+      <c r="AJ20" s="64"/>
+      <c r="AK20" s="64"/>
+      <c r="AL20" s="64"/>
+      <c r="AM20" s="64"/>
+      <c r="AN20" s="64"/>
+      <c r="AO20" s="64"/>
+      <c r="AP20" s="64"/>
       <c r="AQ20" s="11"/>
       <c r="AR20" s="33"/>
       <c r="AS20" s="9"/>
-      <c r="AT20" s="59"/>
-      <c r="AU20" s="59"/>
-      <c r="AV20" s="59"/>
-      <c r="AW20" s="59"/>
-      <c r="AX20" s="59"/>
-      <c r="AY20" s="59"/>
-      <c r="AZ20" s="59"/>
-      <c r="BA20" s="59"/>
-      <c r="BB20" s="59"/>
-      <c r="BC20" s="59"/>
-      <c r="BD20" s="59"/>
-      <c r="BE20" s="59"/>
-      <c r="BF20" s="59"/>
-      <c r="BG20" s="59"/>
-      <c r="BH20" s="59"/>
-      <c r="BI20" s="59"/>
-      <c r="BJ20" s="59"/>
-      <c r="BK20" s="59"/>
-      <c r="BL20" s="59"/>
-      <c r="BM20" s="59"/>
+      <c r="AT20" s="64"/>
+      <c r="AU20" s="64"/>
+      <c r="AV20" s="64"/>
+      <c r="AW20" s="64"/>
+      <c r="AX20" s="64"/>
+      <c r="AY20" s="64"/>
+      <c r="AZ20" s="64"/>
+      <c r="BA20" s="64"/>
+      <c r="BB20" s="64"/>
+      <c r="BC20" s="64"/>
+      <c r="BD20" s="64"/>
+      <c r="BE20" s="64"/>
+      <c r="BF20" s="64"/>
+      <c r="BG20" s="64"/>
+      <c r="BH20" s="64"/>
+      <c r="BI20" s="64"/>
+      <c r="BJ20" s="64"/>
+      <c r="BK20" s="64"/>
+      <c r="BL20" s="64"/>
+      <c r="BM20" s="64"/>
       <c r="BN20" s="24"/>
       <c r="BO20" s="29"/>
-      <c r="BP20" s="59"/>
-      <c r="BQ20" s="59"/>
-      <c r="BR20" s="59"/>
-      <c r="BS20" s="59"/>
-      <c r="BT20" s="59"/>
-      <c r="BU20" s="59"/>
-      <c r="BV20" s="59"/>
+      <c r="BP20" s="64"/>
+      <c r="BQ20" s="64"/>
+      <c r="BR20" s="64"/>
+      <c r="BS20" s="64"/>
+      <c r="BT20" s="64"/>
+      <c r="BU20" s="64"/>
+      <c r="BV20" s="64"/>
       <c r="BW20" s="47"/>
       <c r="BX20" s="24"/>
       <c r="BY20" s="52"/>
-      <c r="BZ20" s="66"/>
-      <c r="CA20" s="66"/>
-      <c r="CB20" s="66"/>
-      <c r="CC20" s="66"/>
-      <c r="CD20" s="66"/>
+      <c r="BZ20" s="71"/>
+      <c r="CA20" s="71"/>
+      <c r="CB20" s="71"/>
+      <c r="CC20" s="71"/>
+      <c r="CD20" s="71"/>
       <c r="CE20" s="48"/>
       <c r="CF20" s="18"/>
       <c r="CG20" s="6"/>
@@ -8480,45 +8480,45 @@
       <c r="AQ46" s="6"/>
       <c r="AR46" s="33"/>
       <c r="AS46" s="5"/>
-      <c r="AT46" s="60" t="s">
+      <c r="AT46" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="AU46" s="60"/>
-      <c r="AV46" s="60"/>
-      <c r="AW46" s="60"/>
-      <c r="AX46" s="60"/>
-      <c r="AY46" s="60"/>
-      <c r="AZ46" s="60"/>
-      <c r="BA46" s="60"/>
-      <c r="BB46" s="60"/>
-      <c r="BC46" s="60"/>
-      <c r="BD46" s="60"/>
-      <c r="BE46" s="60"/>
-      <c r="BF46" s="60"/>
-      <c r="BG46" s="60"/>
-      <c r="BH46" s="60"/>
-      <c r="BI46" s="60"/>
-      <c r="BJ46" s="60"/>
-      <c r="BK46" s="60"/>
-      <c r="BL46" s="60"/>
-      <c r="BM46" s="60"/>
-      <c r="BN46" s="60"/>
-      <c r="BO46" s="60"/>
-      <c r="BP46" s="60"/>
-      <c r="BQ46" s="60"/>
-      <c r="BR46" s="60"/>
-      <c r="BS46" s="60"/>
-      <c r="BT46" s="60"/>
-      <c r="BU46" s="60"/>
-      <c r="BV46" s="60"/>
-      <c r="BW46" s="60"/>
-      <c r="BX46" s="60"/>
-      <c r="BY46" s="60"/>
-      <c r="BZ46" s="60"/>
-      <c r="CA46" s="60"/>
-      <c r="CB46" s="60"/>
-      <c r="CC46" s="60"/>
-      <c r="CD46" s="60"/>
+      <c r="AU46" s="65"/>
+      <c r="AV46" s="65"/>
+      <c r="AW46" s="65"/>
+      <c r="AX46" s="65"/>
+      <c r="AY46" s="65"/>
+      <c r="AZ46" s="65"/>
+      <c r="BA46" s="65"/>
+      <c r="BB46" s="65"/>
+      <c r="BC46" s="65"/>
+      <c r="BD46" s="65"/>
+      <c r="BE46" s="65"/>
+      <c r="BF46" s="65"/>
+      <c r="BG46" s="65"/>
+      <c r="BH46" s="65"/>
+      <c r="BI46" s="65"/>
+      <c r="BJ46" s="65"/>
+      <c r="BK46" s="65"/>
+      <c r="BL46" s="65"/>
+      <c r="BM46" s="65"/>
+      <c r="BN46" s="65"/>
+      <c r="BO46" s="65"/>
+      <c r="BP46" s="65"/>
+      <c r="BQ46" s="65"/>
+      <c r="BR46" s="65"/>
+      <c r="BS46" s="65"/>
+      <c r="BT46" s="65"/>
+      <c r="BU46" s="65"/>
+      <c r="BV46" s="65"/>
+      <c r="BW46" s="65"/>
+      <c r="BX46" s="65"/>
+      <c r="BY46" s="65"/>
+      <c r="BZ46" s="65"/>
+      <c r="CA46" s="65"/>
+      <c r="CB46" s="65"/>
+      <c r="CC46" s="65"/>
+      <c r="CD46" s="65"/>
       <c r="CE46" s="6"/>
       <c r="CF46" s="18"/>
       <c r="CG46" s="6"/>
@@ -8611,45 +8611,45 @@
       <c r="AQ48" s="6"/>
       <c r="AR48" s="33"/>
       <c r="AS48" s="5"/>
-      <c r="AT48" s="71" t="s">
+      <c r="AT48" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="AU48" s="71"/>
-      <c r="AV48" s="71"/>
-      <c r="AW48" s="71"/>
-      <c r="AX48" s="71"/>
-      <c r="AY48" s="71"/>
-      <c r="AZ48" s="71"/>
-      <c r="BA48" s="71"/>
-      <c r="BB48" s="71"/>
-      <c r="BC48" s="71"/>
-      <c r="BD48" s="71"/>
-      <c r="BE48" s="71"/>
-      <c r="BF48" s="71"/>
-      <c r="BG48" s="71"/>
-      <c r="BH48" s="71"/>
-      <c r="BI48" s="71"/>
-      <c r="BJ48" s="71"/>
-      <c r="BK48" s="71"/>
-      <c r="BL48" s="71"/>
-      <c r="BM48" s="71"/>
-      <c r="BN48" s="71"/>
-      <c r="BO48" s="71"/>
-      <c r="BP48" s="71"/>
-      <c r="BQ48" s="71"/>
-      <c r="BR48" s="71"/>
-      <c r="BS48" s="71"/>
-      <c r="BT48" s="71"/>
-      <c r="BU48" s="71"/>
-      <c r="BV48" s="71"/>
-      <c r="BW48" s="71"/>
-      <c r="BX48" s="71"/>
-      <c r="BY48" s="71"/>
-      <c r="BZ48" s="71"/>
-      <c r="CA48" s="71"/>
-      <c r="CB48" s="71"/>
-      <c r="CC48" s="71"/>
-      <c r="CD48" s="71"/>
+      <c r="AU48" s="58"/>
+      <c r="AV48" s="58"/>
+      <c r="AW48" s="58"/>
+      <c r="AX48" s="58"/>
+      <c r="AY48" s="58"/>
+      <c r="AZ48" s="58"/>
+      <c r="BA48" s="58"/>
+      <c r="BB48" s="58"/>
+      <c r="BC48" s="58"/>
+      <c r="BD48" s="58"/>
+      <c r="BE48" s="58"/>
+      <c r="BF48" s="58"/>
+      <c r="BG48" s="58"/>
+      <c r="BH48" s="58"/>
+      <c r="BI48" s="58"/>
+      <c r="BJ48" s="58"/>
+      <c r="BK48" s="58"/>
+      <c r="BL48" s="58"/>
+      <c r="BM48" s="58"/>
+      <c r="BN48" s="58"/>
+      <c r="BO48" s="58"/>
+      <c r="BP48" s="58"/>
+      <c r="BQ48" s="58"/>
+      <c r="BR48" s="58"/>
+      <c r="BS48" s="58"/>
+      <c r="BT48" s="58"/>
+      <c r="BU48" s="58"/>
+      <c r="BV48" s="58"/>
+      <c r="BW48" s="58"/>
+      <c r="BX48" s="58"/>
+      <c r="BY48" s="58"/>
+      <c r="BZ48" s="58"/>
+      <c r="CA48" s="58"/>
+      <c r="CB48" s="58"/>
+      <c r="CC48" s="58"/>
+      <c r="CD48" s="58"/>
       <c r="CE48" s="6"/>
       <c r="CF48" s="18"/>
       <c r="CG48" s="6"/>
@@ -8671,43 +8671,43 @@
       <c r="AQ49" s="6"/>
       <c r="AR49" s="33"/>
       <c r="AS49" s="5"/>
-      <c r="AT49" s="71"/>
-      <c r="AU49" s="71"/>
-      <c r="AV49" s="71"/>
-      <c r="AW49" s="71"/>
-      <c r="AX49" s="71"/>
-      <c r="AY49" s="71"/>
-      <c r="AZ49" s="71"/>
-      <c r="BA49" s="71"/>
-      <c r="BB49" s="71"/>
-      <c r="BC49" s="71"/>
-      <c r="BD49" s="71"/>
-      <c r="BE49" s="71"/>
-      <c r="BF49" s="71"/>
-      <c r="BG49" s="71"/>
-      <c r="BH49" s="71"/>
-      <c r="BI49" s="71"/>
-      <c r="BJ49" s="71"/>
-      <c r="BK49" s="71"/>
-      <c r="BL49" s="71"/>
-      <c r="BM49" s="71"/>
-      <c r="BN49" s="71"/>
-      <c r="BO49" s="71"/>
-      <c r="BP49" s="71"/>
-      <c r="BQ49" s="71"/>
-      <c r="BR49" s="71"/>
-      <c r="BS49" s="71"/>
-      <c r="BT49" s="71"/>
-      <c r="BU49" s="71"/>
-      <c r="BV49" s="71"/>
-      <c r="BW49" s="71"/>
-      <c r="BX49" s="71"/>
-      <c r="BY49" s="71"/>
-      <c r="BZ49" s="71"/>
-      <c r="CA49" s="71"/>
-      <c r="CB49" s="71"/>
-      <c r="CC49" s="71"/>
-      <c r="CD49" s="71"/>
+      <c r="AT49" s="58"/>
+      <c r="AU49" s="58"/>
+      <c r="AV49" s="58"/>
+      <c r="AW49" s="58"/>
+      <c r="AX49" s="58"/>
+      <c r="AY49" s="58"/>
+      <c r="AZ49" s="58"/>
+      <c r="BA49" s="58"/>
+      <c r="BB49" s="58"/>
+      <c r="BC49" s="58"/>
+      <c r="BD49" s="58"/>
+      <c r="BE49" s="58"/>
+      <c r="BF49" s="58"/>
+      <c r="BG49" s="58"/>
+      <c r="BH49" s="58"/>
+      <c r="BI49" s="58"/>
+      <c r="BJ49" s="58"/>
+      <c r="BK49" s="58"/>
+      <c r="BL49" s="58"/>
+      <c r="BM49" s="58"/>
+      <c r="BN49" s="58"/>
+      <c r="BO49" s="58"/>
+      <c r="BP49" s="58"/>
+      <c r="BQ49" s="58"/>
+      <c r="BR49" s="58"/>
+      <c r="BS49" s="58"/>
+      <c r="BT49" s="58"/>
+      <c r="BU49" s="58"/>
+      <c r="BV49" s="58"/>
+      <c r="BW49" s="58"/>
+      <c r="BX49" s="58"/>
+      <c r="BY49" s="58"/>
+      <c r="BZ49" s="58"/>
+      <c r="CA49" s="58"/>
+      <c r="CB49" s="58"/>
+      <c r="CC49" s="58"/>
+      <c r="CD49" s="58"/>
       <c r="CE49" s="6"/>
       <c r="CF49" s="18"/>
       <c r="CG49" s="6"/>
@@ -8779,43 +8779,43 @@
       <c r="AQ50" s="6"/>
       <c r="AR50" s="33"/>
       <c r="AS50" s="5"/>
-      <c r="AT50" s="71"/>
-      <c r="AU50" s="71"/>
-      <c r="AV50" s="71"/>
-      <c r="AW50" s="71"/>
-      <c r="AX50" s="71"/>
-      <c r="AY50" s="71"/>
-      <c r="AZ50" s="71"/>
-      <c r="BA50" s="71"/>
-      <c r="BB50" s="71"/>
-      <c r="BC50" s="71"/>
-      <c r="BD50" s="71"/>
-      <c r="BE50" s="71"/>
-      <c r="BF50" s="71"/>
-      <c r="BG50" s="71"/>
-      <c r="BH50" s="71"/>
-      <c r="BI50" s="71"/>
-      <c r="BJ50" s="71"/>
-      <c r="BK50" s="71"/>
-      <c r="BL50" s="71"/>
-      <c r="BM50" s="71"/>
-      <c r="BN50" s="71"/>
-      <c r="BO50" s="71"/>
-      <c r="BP50" s="71"/>
-      <c r="BQ50" s="71"/>
-      <c r="BR50" s="71"/>
-      <c r="BS50" s="71"/>
-      <c r="BT50" s="71"/>
-      <c r="BU50" s="71"/>
-      <c r="BV50" s="71"/>
-      <c r="BW50" s="71"/>
-      <c r="BX50" s="71"/>
-      <c r="BY50" s="71"/>
-      <c r="BZ50" s="71"/>
-      <c r="CA50" s="71"/>
-      <c r="CB50" s="71"/>
-      <c r="CC50" s="71"/>
-      <c r="CD50" s="71"/>
+      <c r="AT50" s="58"/>
+      <c r="AU50" s="58"/>
+      <c r="AV50" s="58"/>
+      <c r="AW50" s="58"/>
+      <c r="AX50" s="58"/>
+      <c r="AY50" s="58"/>
+      <c r="AZ50" s="58"/>
+      <c r="BA50" s="58"/>
+      <c r="BB50" s="58"/>
+      <c r="BC50" s="58"/>
+      <c r="BD50" s="58"/>
+      <c r="BE50" s="58"/>
+      <c r="BF50" s="58"/>
+      <c r="BG50" s="58"/>
+      <c r="BH50" s="58"/>
+      <c r="BI50" s="58"/>
+      <c r="BJ50" s="58"/>
+      <c r="BK50" s="58"/>
+      <c r="BL50" s="58"/>
+      <c r="BM50" s="58"/>
+      <c r="BN50" s="58"/>
+      <c r="BO50" s="58"/>
+      <c r="BP50" s="58"/>
+      <c r="BQ50" s="58"/>
+      <c r="BR50" s="58"/>
+      <c r="BS50" s="58"/>
+      <c r="BT50" s="58"/>
+      <c r="BU50" s="58"/>
+      <c r="BV50" s="58"/>
+      <c r="BW50" s="58"/>
+      <c r="BX50" s="58"/>
+      <c r="BY50" s="58"/>
+      <c r="BZ50" s="58"/>
+      <c r="CA50" s="58"/>
+      <c r="CB50" s="58"/>
+      <c r="CC50" s="58"/>
+      <c r="CD50" s="58"/>
       <c r="CE50" s="6"/>
       <c r="CF50" s="18"/>
       <c r="CG50" s="6"/>
@@ -8840,43 +8840,43 @@
       <c r="AQ51" s="6"/>
       <c r="AR51" s="33"/>
       <c r="AS51" s="5"/>
-      <c r="AT51" s="71"/>
-      <c r="AU51" s="71"/>
-      <c r="AV51" s="71"/>
-      <c r="AW51" s="71"/>
-      <c r="AX51" s="71"/>
-      <c r="AY51" s="71"/>
-      <c r="AZ51" s="71"/>
-      <c r="BA51" s="71"/>
-      <c r="BB51" s="71"/>
-      <c r="BC51" s="71"/>
-      <c r="BD51" s="71"/>
-      <c r="BE51" s="71"/>
-      <c r="BF51" s="71"/>
-      <c r="BG51" s="71"/>
-      <c r="BH51" s="71"/>
-      <c r="BI51" s="71"/>
-      <c r="BJ51" s="71"/>
-      <c r="BK51" s="71"/>
-      <c r="BL51" s="71"/>
-      <c r="BM51" s="71"/>
-      <c r="BN51" s="71"/>
-      <c r="BO51" s="71"/>
-      <c r="BP51" s="71"/>
-      <c r="BQ51" s="71"/>
-      <c r="BR51" s="71"/>
-      <c r="BS51" s="71"/>
-      <c r="BT51" s="71"/>
-      <c r="BU51" s="71"/>
-      <c r="BV51" s="71"/>
-      <c r="BW51" s="71"/>
-      <c r="BX51" s="71"/>
-      <c r="BY51" s="71"/>
-      <c r="BZ51" s="71"/>
-      <c r="CA51" s="71"/>
-      <c r="CB51" s="71"/>
-      <c r="CC51" s="71"/>
-      <c r="CD51" s="71"/>
+      <c r="AT51" s="58"/>
+      <c r="AU51" s="58"/>
+      <c r="AV51" s="58"/>
+      <c r="AW51" s="58"/>
+      <c r="AX51" s="58"/>
+      <c r="AY51" s="58"/>
+      <c r="AZ51" s="58"/>
+      <c r="BA51" s="58"/>
+      <c r="BB51" s="58"/>
+      <c r="BC51" s="58"/>
+      <c r="BD51" s="58"/>
+      <c r="BE51" s="58"/>
+      <c r="BF51" s="58"/>
+      <c r="BG51" s="58"/>
+      <c r="BH51" s="58"/>
+      <c r="BI51" s="58"/>
+      <c r="BJ51" s="58"/>
+      <c r="BK51" s="58"/>
+      <c r="BL51" s="58"/>
+      <c r="BM51" s="58"/>
+      <c r="BN51" s="58"/>
+      <c r="BO51" s="58"/>
+      <c r="BP51" s="58"/>
+      <c r="BQ51" s="58"/>
+      <c r="BR51" s="58"/>
+      <c r="BS51" s="58"/>
+      <c r="BT51" s="58"/>
+      <c r="BU51" s="58"/>
+      <c r="BV51" s="58"/>
+      <c r="BW51" s="58"/>
+      <c r="BX51" s="58"/>
+      <c r="BY51" s="58"/>
+      <c r="BZ51" s="58"/>
+      <c r="CA51" s="58"/>
+      <c r="CB51" s="58"/>
+      <c r="CC51" s="58"/>
+      <c r="CD51" s="58"/>
       <c r="CE51" s="6"/>
       <c r="CF51" s="18"/>
       <c r="CG51" s="6"/>
@@ -8948,43 +8948,43 @@
       <c r="AQ52" s="6"/>
       <c r="AR52" s="33"/>
       <c r="AS52" s="5"/>
-      <c r="AT52" s="71"/>
-      <c r="AU52" s="71"/>
-      <c r="AV52" s="71"/>
-      <c r="AW52" s="71"/>
-      <c r="AX52" s="71"/>
-      <c r="AY52" s="71"/>
-      <c r="AZ52" s="71"/>
-      <c r="BA52" s="71"/>
-      <c r="BB52" s="71"/>
-      <c r="BC52" s="71"/>
-      <c r="BD52" s="71"/>
-      <c r="BE52" s="71"/>
-      <c r="BF52" s="71"/>
-      <c r="BG52" s="71"/>
-      <c r="BH52" s="71"/>
-      <c r="BI52" s="71"/>
-      <c r="BJ52" s="71"/>
-      <c r="BK52" s="71"/>
-      <c r="BL52" s="71"/>
-      <c r="BM52" s="71"/>
-      <c r="BN52" s="71"/>
-      <c r="BO52" s="71"/>
-      <c r="BP52" s="71"/>
-      <c r="BQ52" s="71"/>
-      <c r="BR52" s="71"/>
-      <c r="BS52" s="71"/>
-      <c r="BT52" s="71"/>
-      <c r="BU52" s="71"/>
-      <c r="BV52" s="71"/>
-      <c r="BW52" s="71"/>
-      <c r="BX52" s="71"/>
-      <c r="BY52" s="71"/>
-      <c r="BZ52" s="71"/>
-      <c r="CA52" s="71"/>
-      <c r="CB52" s="71"/>
-      <c r="CC52" s="71"/>
-      <c r="CD52" s="71"/>
+      <c r="AT52" s="58"/>
+      <c r="AU52" s="58"/>
+      <c r="AV52" s="58"/>
+      <c r="AW52" s="58"/>
+      <c r="AX52" s="58"/>
+      <c r="AY52" s="58"/>
+      <c r="AZ52" s="58"/>
+      <c r="BA52" s="58"/>
+      <c r="BB52" s="58"/>
+      <c r="BC52" s="58"/>
+      <c r="BD52" s="58"/>
+      <c r="BE52" s="58"/>
+      <c r="BF52" s="58"/>
+      <c r="BG52" s="58"/>
+      <c r="BH52" s="58"/>
+      <c r="BI52" s="58"/>
+      <c r="BJ52" s="58"/>
+      <c r="BK52" s="58"/>
+      <c r="BL52" s="58"/>
+      <c r="BM52" s="58"/>
+      <c r="BN52" s="58"/>
+      <c r="BO52" s="58"/>
+      <c r="BP52" s="58"/>
+      <c r="BQ52" s="58"/>
+      <c r="BR52" s="58"/>
+      <c r="BS52" s="58"/>
+      <c r="BT52" s="58"/>
+      <c r="BU52" s="58"/>
+      <c r="BV52" s="58"/>
+      <c r="BW52" s="58"/>
+      <c r="BX52" s="58"/>
+      <c r="BY52" s="58"/>
+      <c r="BZ52" s="58"/>
+      <c r="CA52" s="58"/>
+      <c r="CB52" s="58"/>
+      <c r="CC52" s="58"/>
+      <c r="CD52" s="58"/>
       <c r="CE52" s="6"/>
       <c r="CF52" s="18"/>
       <c r="CG52" s="6"/>
@@ -9077,45 +9077,45 @@
       <c r="AQ54" s="6"/>
       <c r="AR54" s="33"/>
       <c r="AS54" s="9"/>
-      <c r="AT54" s="68" t="s">
+      <c r="AT54" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="AU54" s="68"/>
-      <c r="AV54" s="68"/>
-      <c r="AW54" s="68"/>
-      <c r="AX54" s="68"/>
-      <c r="AY54" s="68"/>
-      <c r="AZ54" s="68"/>
-      <c r="BA54" s="68"/>
-      <c r="BB54" s="68"/>
-      <c r="BC54" s="68"/>
-      <c r="BD54" s="68"/>
-      <c r="BE54" s="68"/>
-      <c r="BF54" s="68"/>
-      <c r="BG54" s="68"/>
-      <c r="BH54" s="68"/>
-      <c r="BI54" s="68"/>
-      <c r="BJ54" s="68"/>
-      <c r="BK54" s="68"/>
-      <c r="BL54" s="68"/>
-      <c r="BM54" s="68"/>
-      <c r="BN54" s="68"/>
-      <c r="BO54" s="68"/>
-      <c r="BP54" s="68"/>
-      <c r="BQ54" s="68"/>
-      <c r="BR54" s="68"/>
-      <c r="BS54" s="68"/>
-      <c r="BT54" s="68"/>
-      <c r="BU54" s="68"/>
-      <c r="BV54" s="68"/>
-      <c r="BW54" s="68"/>
-      <c r="BX54" s="68"/>
-      <c r="BY54" s="68"/>
-      <c r="BZ54" s="68"/>
-      <c r="CA54" s="68"/>
-      <c r="CB54" s="68"/>
-      <c r="CC54" s="68"/>
-      <c r="CD54" s="68"/>
+      <c r="AU54" s="57"/>
+      <c r="AV54" s="57"/>
+      <c r="AW54" s="57"/>
+      <c r="AX54" s="57"/>
+      <c r="AY54" s="57"/>
+      <c r="AZ54" s="57"/>
+      <c r="BA54" s="57"/>
+      <c r="BB54" s="57"/>
+      <c r="BC54" s="57"/>
+      <c r="BD54" s="57"/>
+      <c r="BE54" s="57"/>
+      <c r="BF54" s="57"/>
+      <c r="BG54" s="57"/>
+      <c r="BH54" s="57"/>
+      <c r="BI54" s="57"/>
+      <c r="BJ54" s="57"/>
+      <c r="BK54" s="57"/>
+      <c r="BL54" s="57"/>
+      <c r="BM54" s="57"/>
+      <c r="BN54" s="57"/>
+      <c r="BO54" s="57"/>
+      <c r="BP54" s="57"/>
+      <c r="BQ54" s="57"/>
+      <c r="BR54" s="57"/>
+      <c r="BS54" s="57"/>
+      <c r="BT54" s="57"/>
+      <c r="BU54" s="57"/>
+      <c r="BV54" s="57"/>
+      <c r="BW54" s="57"/>
+      <c r="BX54" s="57"/>
+      <c r="BY54" s="57"/>
+      <c r="BZ54" s="57"/>
+      <c r="CA54" s="57"/>
+      <c r="CB54" s="57"/>
+      <c r="CC54" s="57"/>
+      <c r="CD54" s="57"/>
       <c r="CE54" s="11"/>
       <c r="CF54" s="18"/>
       <c r="CG54" s="6"/>
@@ -9704,45 +9704,45 @@
       <c r="AQ62" s="6"/>
       <c r="AR62" s="33"/>
       <c r="AS62" s="9"/>
-      <c r="AT62" s="68" t="s">
+      <c r="AT62" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="AU62" s="68"/>
-      <c r="AV62" s="68"/>
-      <c r="AW62" s="68"/>
-      <c r="AX62" s="68"/>
-      <c r="AY62" s="68"/>
-      <c r="AZ62" s="68"/>
-      <c r="BA62" s="68"/>
-      <c r="BB62" s="68"/>
-      <c r="BC62" s="68"/>
-      <c r="BD62" s="68"/>
-      <c r="BE62" s="68"/>
-      <c r="BF62" s="68"/>
-      <c r="BG62" s="68"/>
-      <c r="BH62" s="68"/>
-      <c r="BI62" s="68"/>
-      <c r="BJ62" s="68"/>
-      <c r="BK62" s="68"/>
-      <c r="BL62" s="68"/>
-      <c r="BM62" s="68"/>
-      <c r="BN62" s="68"/>
-      <c r="BO62" s="68"/>
-      <c r="BP62" s="68"/>
-      <c r="BQ62" s="68"/>
-      <c r="BR62" s="68"/>
-      <c r="BS62" s="68"/>
-      <c r="BT62" s="68"/>
-      <c r="BU62" s="68"/>
-      <c r="BV62" s="68"/>
-      <c r="BW62" s="68"/>
-      <c r="BX62" s="68"/>
-      <c r="BY62" s="68"/>
-      <c r="BZ62" s="68"/>
-      <c r="CA62" s="68"/>
-      <c r="CB62" s="68"/>
-      <c r="CC62" s="68"/>
-      <c r="CD62" s="68"/>
+      <c r="AU62" s="57"/>
+      <c r="AV62" s="57"/>
+      <c r="AW62" s="57"/>
+      <c r="AX62" s="57"/>
+      <c r="AY62" s="57"/>
+      <c r="AZ62" s="57"/>
+      <c r="BA62" s="57"/>
+      <c r="BB62" s="57"/>
+      <c r="BC62" s="57"/>
+      <c r="BD62" s="57"/>
+      <c r="BE62" s="57"/>
+      <c r="BF62" s="57"/>
+      <c r="BG62" s="57"/>
+      <c r="BH62" s="57"/>
+      <c r="BI62" s="57"/>
+      <c r="BJ62" s="57"/>
+      <c r="BK62" s="57"/>
+      <c r="BL62" s="57"/>
+      <c r="BM62" s="57"/>
+      <c r="BN62" s="57"/>
+      <c r="BO62" s="57"/>
+      <c r="BP62" s="57"/>
+      <c r="BQ62" s="57"/>
+      <c r="BR62" s="57"/>
+      <c r="BS62" s="57"/>
+      <c r="BT62" s="57"/>
+      <c r="BU62" s="57"/>
+      <c r="BV62" s="57"/>
+      <c r="BW62" s="57"/>
+      <c r="BX62" s="57"/>
+      <c r="BY62" s="57"/>
+      <c r="BZ62" s="57"/>
+      <c r="CA62" s="57"/>
+      <c r="CB62" s="57"/>
+      <c r="CC62" s="57"/>
+      <c r="CD62" s="57"/>
       <c r="CE62" s="11"/>
       <c r="CF62" s="18"/>
       <c r="CG62" s="6"/>
@@ -9835,10 +9835,10 @@
       <c r="AQ64" s="6"/>
       <c r="AR64" s="33"/>
       <c r="AS64" s="5"/>
-      <c r="AU64" s="67">
+      <c r="AU64" s="56">
         <v>1</v>
       </c>
-      <c r="AV64" s="67"/>
+      <c r="AV64" s="56"/>
       <c r="AX64" s="7" t="s">
         <v>2</v>
       </c>
@@ -9854,10 +9854,10 @@
       <c r="BD64" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BG64" s="67">
+      <c r="BG64" s="56">
         <v>6</v>
       </c>
-      <c r="BH64" s="67"/>
+      <c r="BH64" s="56"/>
       <c r="BJ64" s="7" t="s">
         <v>2</v>
       </c>
@@ -9873,10 +9873,10 @@
       <c r="BP64" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BS64" s="67">
+      <c r="BS64" s="56">
         <v>11</v>
       </c>
-      <c r="BT64" s="67"/>
+      <c r="BT64" s="56"/>
       <c r="BV64" s="7" t="s">
         <v>2</v>
       </c>
@@ -9984,10 +9984,10 @@
       <c r="AQ66" s="6"/>
       <c r="AR66" s="33"/>
       <c r="AS66" s="5"/>
-      <c r="AU66" s="67">
+      <c r="AU66" s="56">
         <v>2</v>
       </c>
-      <c r="AV66" s="67"/>
+      <c r="AV66" s="56"/>
       <c r="AX66" s="7" t="s">
         <v>2</v>
       </c>
@@ -10003,10 +10003,10 @@
       <c r="BD66" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BG66" s="67">
+      <c r="BG66" s="56">
         <v>7</v>
       </c>
-      <c r="BH66" s="67"/>
+      <c r="BH66" s="56"/>
       <c r="BJ66" s="7" t="s">
         <v>2</v>
       </c>
@@ -10022,10 +10022,10 @@
       <c r="BP66" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BS66" s="67">
+      <c r="BS66" s="56">
         <v>12</v>
       </c>
-      <c r="BT66" s="67"/>
+      <c r="BT66" s="56"/>
       <c r="BV66" s="7" t="s">
         <v>2</v>
       </c>
@@ -10133,10 +10133,10 @@
       <c r="AQ68" s="6"/>
       <c r="AR68" s="33"/>
       <c r="AS68" s="5"/>
-      <c r="AU68" s="67">
+      <c r="AU68" s="56">
         <v>3</v>
       </c>
-      <c r="AV68" s="67"/>
+      <c r="AV68" s="56"/>
       <c r="AX68" s="7" t="s">
         <v>2</v>
       </c>
@@ -10152,10 +10152,10 @@
       <c r="BD68" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BG68" s="67">
+      <c r="BG68" s="56">
         <v>8</v>
       </c>
-      <c r="BH68" s="67"/>
+      <c r="BH68" s="56"/>
       <c r="BJ68" s="7" t="s">
         <v>2</v>
       </c>
@@ -10171,10 +10171,10 @@
       <c r="BP68" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BS68" s="67">
+      <c r="BS68" s="56">
         <v>13</v>
       </c>
-      <c r="BT68" s="67"/>
+      <c r="BT68" s="56"/>
       <c r="BV68" s="7" t="s">
         <v>2</v>
       </c>
@@ -10282,10 +10282,10 @@
       <c r="AQ70" s="6"/>
       <c r="AR70" s="33"/>
       <c r="AS70" s="5"/>
-      <c r="AU70" s="67">
+      <c r="AU70" s="56">
         <v>4</v>
       </c>
-      <c r="AV70" s="67"/>
+      <c r="AV70" s="56"/>
       <c r="AX70" s="7" t="s">
         <v>2</v>
       </c>
@@ -10301,10 +10301,10 @@
       <c r="BD70" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BG70" s="67">
+      <c r="BG70" s="56">
         <v>9</v>
       </c>
-      <c r="BH70" s="67"/>
+      <c r="BH70" s="56"/>
       <c r="BJ70" s="7" t="s">
         <v>2</v>
       </c>
@@ -10320,10 +10320,10 @@
       <c r="BP70" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BS70" s="67">
+      <c r="BS70" s="56">
         <v>14</v>
       </c>
-      <c r="BT70" s="67"/>
+      <c r="BT70" s="56"/>
       <c r="BV70" s="7" t="s">
         <v>2</v>
       </c>
@@ -10360,8 +10360,8 @@
       <c r="AQ71" s="6"/>
       <c r="AR71" s="33"/>
       <c r="AS71" s="5"/>
-      <c r="AU71" s="67"/>
-      <c r="AV71" s="67"/>
+      <c r="AU71" s="56"/>
+      <c r="AV71" s="56"/>
       <c r="CE71" s="6"/>
       <c r="CF71" s="18"/>
       <c r="CG71" s="6"/>
@@ -10433,10 +10433,10 @@
       <c r="AQ72" s="6"/>
       <c r="AR72" s="33"/>
       <c r="AS72" s="5"/>
-      <c r="AU72" s="67">
+      <c r="AU72" s="56">
         <v>5</v>
       </c>
-      <c r="AV72" s="67"/>
+      <c r="AV72" s="56"/>
       <c r="AX72" s="7" t="s">
         <v>2</v>
       </c>
@@ -10452,10 +10452,10 @@
       <c r="BD72" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BG72" s="67">
+      <c r="BG72" s="56">
         <v>10</v>
       </c>
-      <c r="BH72" s="67"/>
+      <c r="BH72" s="56"/>
       <c r="BJ72" s="7" t="s">
         <v>2</v>
       </c>
@@ -10471,10 +10471,10 @@
       <c r="BP72" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BS72" s="67">
+      <c r="BS72" s="56">
         <v>15</v>
       </c>
-      <c r="BT72" s="67"/>
+      <c r="BT72" s="56"/>
       <c r="BV72" s="7" t="s">
         <v>2</v>
       </c>
@@ -10494,7 +10494,7 @@
       <c r="CF72" s="18"/>
       <c r="CG72" s="6"/>
     </row>
-    <row r="73" spans="1:85" ht="7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="5"/>
       <c r="B73" s="20"/>
       <c r="C73" s="5"/>
@@ -10801,87 +10801,87 @@
       <c r="A77" s="5"/>
       <c r="B77" s="20"/>
       <c r="C77" s="1"/>
-      <c r="D77" s="69" t="s">
+      <c r="D77" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="E77" s="69"/>
-      <c r="F77" s="69"/>
-      <c r="G77" s="69"/>
-      <c r="H77" s="69"/>
-      <c r="I77" s="69"/>
-      <c r="J77" s="69"/>
-      <c r="K77" s="69"/>
-      <c r="L77" s="69"/>
-      <c r="M77" s="69"/>
-      <c r="N77" s="69"/>
-      <c r="O77" s="69"/>
-      <c r="P77" s="69"/>
-      <c r="Q77" s="69"/>
-      <c r="R77" s="69"/>
-      <c r="S77" s="69"/>
-      <c r="T77" s="69"/>
-      <c r="U77" s="69"/>
-      <c r="V77" s="69"/>
-      <c r="W77" s="69"/>
-      <c r="X77" s="69"/>
-      <c r="Y77" s="69"/>
-      <c r="Z77" s="69"/>
-      <c r="AA77" s="69"/>
-      <c r="AB77" s="69"/>
-      <c r="AC77" s="69"/>
-      <c r="AD77" s="69"/>
-      <c r="AE77" s="69"/>
-      <c r="AF77" s="69"/>
-      <c r="AG77" s="69"/>
-      <c r="AH77" s="69"/>
-      <c r="AI77" s="69"/>
-      <c r="AJ77" s="69"/>
-      <c r="AK77" s="69"/>
-      <c r="AL77" s="69"/>
-      <c r="AM77" s="69"/>
-      <c r="AN77" s="69"/>
-      <c r="AO77" s="69"/>
-      <c r="AP77" s="69"/>
-      <c r="AQ77" s="69"/>
-      <c r="AR77" s="69"/>
-      <c r="AS77" s="69"/>
-      <c r="AT77" s="69"/>
-      <c r="AU77" s="69"/>
-      <c r="AV77" s="69"/>
-      <c r="AW77" s="69"/>
-      <c r="AX77" s="69"/>
-      <c r="AY77" s="69"/>
-      <c r="AZ77" s="69"/>
-      <c r="BA77" s="69"/>
-      <c r="BB77" s="69"/>
-      <c r="BC77" s="69"/>
-      <c r="BD77" s="69"/>
-      <c r="BE77" s="69"/>
-      <c r="BF77" s="69"/>
-      <c r="BG77" s="69"/>
-      <c r="BH77" s="69"/>
-      <c r="BI77" s="69"/>
-      <c r="BJ77" s="69"/>
-      <c r="BK77" s="69"/>
-      <c r="BL77" s="69"/>
-      <c r="BM77" s="69"/>
-      <c r="BN77" s="69"/>
-      <c r="BO77" s="69"/>
-      <c r="BP77" s="69"/>
-      <c r="BQ77" s="69"/>
-      <c r="BR77" s="69"/>
-      <c r="BS77" s="69"/>
-      <c r="BT77" s="69"/>
-      <c r="BU77" s="69"/>
-      <c r="BV77" s="69"/>
-      <c r="BW77" s="69"/>
-      <c r="BX77" s="69"/>
-      <c r="BY77" s="69"/>
-      <c r="BZ77" s="69"/>
-      <c r="CA77" s="69"/>
-      <c r="CB77" s="69"/>
-      <c r="CC77" s="69"/>
-      <c r="CD77" s="69"/>
+      <c r="E77" s="60"/>
+      <c r="F77" s="60"/>
+      <c r="G77" s="60"/>
+      <c r="H77" s="60"/>
+      <c r="I77" s="60"/>
+      <c r="J77" s="60"/>
+      <c r="K77" s="60"/>
+      <c r="L77" s="60"/>
+      <c r="M77" s="60"/>
+      <c r="N77" s="60"/>
+      <c r="O77" s="60"/>
+      <c r="P77" s="60"/>
+      <c r="Q77" s="60"/>
+      <c r="R77" s="60"/>
+      <c r="S77" s="60"/>
+      <c r="T77" s="60"/>
+      <c r="U77" s="60"/>
+      <c r="V77" s="60"/>
+      <c r="W77" s="60"/>
+      <c r="X77" s="60"/>
+      <c r="Y77" s="60"/>
+      <c r="Z77" s="60"/>
+      <c r="AA77" s="60"/>
+      <c r="AB77" s="60"/>
+      <c r="AC77" s="60"/>
+      <c r="AD77" s="60"/>
+      <c r="AE77" s="60"/>
+      <c r="AF77" s="60"/>
+      <c r="AG77" s="60"/>
+      <c r="AH77" s="60"/>
+      <c r="AI77" s="60"/>
+      <c r="AJ77" s="60"/>
+      <c r="AK77" s="60"/>
+      <c r="AL77" s="60"/>
+      <c r="AM77" s="60"/>
+      <c r="AN77" s="60"/>
+      <c r="AO77" s="60"/>
+      <c r="AP77" s="60"/>
+      <c r="AQ77" s="60"/>
+      <c r="AR77" s="60"/>
+      <c r="AS77" s="60"/>
+      <c r="AT77" s="60"/>
+      <c r="AU77" s="60"/>
+      <c r="AV77" s="60"/>
+      <c r="AW77" s="60"/>
+      <c r="AX77" s="60"/>
+      <c r="AY77" s="60"/>
+      <c r="AZ77" s="60"/>
+      <c r="BA77" s="60"/>
+      <c r="BB77" s="60"/>
+      <c r="BC77" s="60"/>
+      <c r="BD77" s="60"/>
+      <c r="BE77" s="60"/>
+      <c r="BF77" s="60"/>
+      <c r="BG77" s="60"/>
+      <c r="BH77" s="60"/>
+      <c r="BI77" s="60"/>
+      <c r="BJ77" s="60"/>
+      <c r="BK77" s="60"/>
+      <c r="BL77" s="60"/>
+      <c r="BM77" s="60"/>
+      <c r="BN77" s="60"/>
+      <c r="BO77" s="60"/>
+      <c r="BP77" s="60"/>
+      <c r="BQ77" s="60"/>
+      <c r="BR77" s="60"/>
+      <c r="BS77" s="60"/>
+      <c r="BT77" s="60"/>
+      <c r="BU77" s="60"/>
+      <c r="BV77" s="60"/>
+      <c r="BW77" s="60"/>
+      <c r="BX77" s="60"/>
+      <c r="BY77" s="60"/>
+      <c r="BZ77" s="60"/>
+      <c r="CA77" s="60"/>
+      <c r="CB77" s="60"/>
+      <c r="CC77" s="60"/>
+      <c r="CD77" s="60"/>
       <c r="CE77" s="3"/>
       <c r="CF77" s="18"/>
       <c r="CG77" s="6"/>
@@ -10890,87 +10890,87 @@
       <c r="A78" s="5"/>
       <c r="B78" s="20"/>
       <c r="C78" s="9"/>
-      <c r="D78" s="70" t="s">
+      <c r="D78" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="E78" s="70"/>
-      <c r="F78" s="70"/>
-      <c r="G78" s="70"/>
-      <c r="H78" s="70"/>
-      <c r="I78" s="70"/>
-      <c r="J78" s="70"/>
-      <c r="K78" s="70"/>
-      <c r="L78" s="70"/>
-      <c r="M78" s="70"/>
-      <c r="N78" s="70"/>
-      <c r="O78" s="70"/>
-      <c r="P78" s="70"/>
-      <c r="Q78" s="70"/>
-      <c r="R78" s="70"/>
-      <c r="S78" s="70"/>
-      <c r="T78" s="70"/>
-      <c r="U78" s="70"/>
-      <c r="V78" s="70"/>
-      <c r="W78" s="70"/>
-      <c r="X78" s="70"/>
-      <c r="Y78" s="70"/>
-      <c r="Z78" s="70"/>
-      <c r="AA78" s="70"/>
-      <c r="AB78" s="70"/>
-      <c r="AC78" s="70"/>
-      <c r="AD78" s="70"/>
-      <c r="AE78" s="70"/>
-      <c r="AF78" s="70"/>
-      <c r="AG78" s="70"/>
-      <c r="AH78" s="70"/>
-      <c r="AI78" s="70"/>
-      <c r="AJ78" s="70"/>
-      <c r="AK78" s="70"/>
-      <c r="AL78" s="70"/>
-      <c r="AM78" s="70"/>
-      <c r="AN78" s="70"/>
-      <c r="AO78" s="70"/>
-      <c r="AP78" s="70"/>
-      <c r="AQ78" s="70"/>
-      <c r="AR78" s="70"/>
-      <c r="AS78" s="70"/>
-      <c r="AT78" s="70"/>
-      <c r="AU78" s="70"/>
-      <c r="AV78" s="70"/>
-      <c r="AW78" s="70"/>
-      <c r="AX78" s="70"/>
-      <c r="AY78" s="70"/>
-      <c r="AZ78" s="70"/>
-      <c r="BA78" s="70"/>
-      <c r="BB78" s="70"/>
-      <c r="BC78" s="70"/>
-      <c r="BD78" s="70"/>
-      <c r="BE78" s="70"/>
-      <c r="BF78" s="70"/>
-      <c r="BG78" s="70"/>
-      <c r="BH78" s="70"/>
-      <c r="BI78" s="70"/>
-      <c r="BJ78" s="70"/>
-      <c r="BK78" s="70"/>
-      <c r="BL78" s="70"/>
-      <c r="BM78" s="70"/>
-      <c r="BN78" s="70"/>
-      <c r="BO78" s="70"/>
-      <c r="BP78" s="70"/>
-      <c r="BQ78" s="70"/>
-      <c r="BR78" s="70"/>
-      <c r="BS78" s="70"/>
-      <c r="BT78" s="70"/>
-      <c r="BU78" s="70"/>
-      <c r="BV78" s="70"/>
-      <c r="BW78" s="70"/>
-      <c r="BX78" s="70"/>
-      <c r="BY78" s="70"/>
-      <c r="BZ78" s="70"/>
-      <c r="CA78" s="70"/>
-      <c r="CB78" s="70"/>
-      <c r="CC78" s="70"/>
-      <c r="CD78" s="70"/>
+      <c r="E78" s="59"/>
+      <c r="F78" s="59"/>
+      <c r="G78" s="59"/>
+      <c r="H78" s="59"/>
+      <c r="I78" s="59"/>
+      <c r="J78" s="59"/>
+      <c r="K78" s="59"/>
+      <c r="L78" s="59"/>
+      <c r="M78" s="59"/>
+      <c r="N78" s="59"/>
+      <c r="O78" s="59"/>
+      <c r="P78" s="59"/>
+      <c r="Q78" s="59"/>
+      <c r="R78" s="59"/>
+      <c r="S78" s="59"/>
+      <c r="T78" s="59"/>
+      <c r="U78" s="59"/>
+      <c r="V78" s="59"/>
+      <c r="W78" s="59"/>
+      <c r="X78" s="59"/>
+      <c r="Y78" s="59"/>
+      <c r="Z78" s="59"/>
+      <c r="AA78" s="59"/>
+      <c r="AB78" s="59"/>
+      <c r="AC78" s="59"/>
+      <c r="AD78" s="59"/>
+      <c r="AE78" s="59"/>
+      <c r="AF78" s="59"/>
+      <c r="AG78" s="59"/>
+      <c r="AH78" s="59"/>
+      <c r="AI78" s="59"/>
+      <c r="AJ78" s="59"/>
+      <c r="AK78" s="59"/>
+      <c r="AL78" s="59"/>
+      <c r="AM78" s="59"/>
+      <c r="AN78" s="59"/>
+      <c r="AO78" s="59"/>
+      <c r="AP78" s="59"/>
+      <c r="AQ78" s="59"/>
+      <c r="AR78" s="59"/>
+      <c r="AS78" s="59"/>
+      <c r="AT78" s="59"/>
+      <c r="AU78" s="59"/>
+      <c r="AV78" s="59"/>
+      <c r="AW78" s="59"/>
+      <c r="AX78" s="59"/>
+      <c r="AY78" s="59"/>
+      <c r="AZ78" s="59"/>
+      <c r="BA78" s="59"/>
+      <c r="BB78" s="59"/>
+      <c r="BC78" s="59"/>
+      <c r="BD78" s="59"/>
+      <c r="BE78" s="59"/>
+      <c r="BF78" s="59"/>
+      <c r="BG78" s="59"/>
+      <c r="BH78" s="59"/>
+      <c r="BI78" s="59"/>
+      <c r="BJ78" s="59"/>
+      <c r="BK78" s="59"/>
+      <c r="BL78" s="59"/>
+      <c r="BM78" s="59"/>
+      <c r="BN78" s="59"/>
+      <c r="BO78" s="59"/>
+      <c r="BP78" s="59"/>
+      <c r="BQ78" s="59"/>
+      <c r="BR78" s="59"/>
+      <c r="BS78" s="59"/>
+      <c r="BT78" s="59"/>
+      <c r="BU78" s="59"/>
+      <c r="BV78" s="59"/>
+      <c r="BW78" s="59"/>
+      <c r="BX78" s="59"/>
+      <c r="BY78" s="59"/>
+      <c r="BZ78" s="59"/>
+      <c r="CA78" s="59"/>
+      <c r="CB78" s="59"/>
+      <c r="CC78" s="59"/>
+      <c r="CD78" s="59"/>
       <c r="CE78" s="11"/>
       <c r="CF78" s="18"/>
       <c r="CG78" s="6"/>
@@ -10987,10 +10987,10 @@
       <c r="A80" s="5"/>
       <c r="B80" s="20"/>
       <c r="C80" s="5"/>
-      <c r="G80" s="67">
+      <c r="G80" s="56">
         <v>1</v>
       </c>
-      <c r="H80" s="67"/>
+      <c r="H80" s="56"/>
       <c r="I80" s="44" t="s">
         <v>31</v>
       </c>
@@ -11029,10 +11029,10 @@
       <c r="AF80" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM80" s="67">
+      <c r="AM80" s="56">
         <v>31</v>
       </c>
-      <c r="AN80" s="67">
+      <c r="AN80" s="56">
         <v>31</v>
       </c>
       <c r="AO80" s="44"/>
@@ -11051,10 +11051,10 @@
       <c r="AV80" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC80" s="67">
+      <c r="BC80" s="56">
         <v>46</v>
       </c>
-      <c r="BD80" s="67">
+      <c r="BD80" s="56">
         <v>46</v>
       </c>
       <c r="BE80" s="44"/>
@@ -11074,10 +11074,10 @@
         <v>5</v>
       </c>
       <c r="BQ80" s="36"/>
-      <c r="BS80" s="67">
+      <c r="BS80" s="56">
         <v>61</v>
       </c>
-      <c r="BT80" s="67">
+      <c r="BT80" s="56">
         <v>41</v>
       </c>
       <c r="BU80" s="44"/>
@@ -11100,7 +11100,7 @@
       <c r="CF80" s="18"/>
       <c r="CG80" s="6"/>
     </row>
-    <row r="81" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="5"/>
       <c r="B81" s="20"/>
       <c r="C81" s="5"/>
@@ -11117,10 +11117,10 @@
       <c r="A82" s="5"/>
       <c r="B82" s="20"/>
       <c r="C82" s="5"/>
-      <c r="G82" s="67">
+      <c r="G82" s="56">
         <v>2</v>
       </c>
-      <c r="H82" s="67"/>
+      <c r="H82" s="56"/>
       <c r="I82" s="44" t="s">
         <v>31</v>
       </c>
@@ -11159,10 +11159,10 @@
       <c r="AF82" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM82" s="67">
+      <c r="AM82" s="56">
         <v>32</v>
       </c>
-      <c r="AN82" s="67">
+      <c r="AN82" s="56">
         <v>32</v>
       </c>
       <c r="AO82" s="44"/>
@@ -11181,10 +11181,10 @@
       <c r="AV82" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC82" s="67">
+      <c r="BC82" s="56">
         <v>47</v>
       </c>
-      <c r="BD82" s="67">
+      <c r="BD82" s="56">
         <v>47</v>
       </c>
       <c r="BE82" s="44"/>
@@ -11204,10 +11204,10 @@
         <v>5</v>
       </c>
       <c r="BQ82" s="36"/>
-      <c r="BS82" s="67">
+      <c r="BS82" s="56">
         <v>62</v>
       </c>
-      <c r="BT82" s="67">
+      <c r="BT82" s="56">
         <v>42</v>
       </c>
       <c r="BU82" s="44"/>
@@ -11230,7 +11230,7 @@
       <c r="CF82" s="18"/>
       <c r="CG82" s="6"/>
     </row>
-    <row r="83" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="5"/>
       <c r="B83" s="20"/>
       <c r="C83" s="5"/>
@@ -11247,10 +11247,10 @@
       <c r="A84" s="5"/>
       <c r="B84" s="20"/>
       <c r="C84" s="5"/>
-      <c r="G84" s="67">
+      <c r="G84" s="56">
         <v>3</v>
       </c>
-      <c r="H84" s="67"/>
+      <c r="H84" s="56"/>
       <c r="I84" s="44" t="s">
         <v>31</v>
       </c>
@@ -11289,10 +11289,10 @@
       <c r="AF84" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM84" s="67">
+      <c r="AM84" s="56">
         <v>33</v>
       </c>
-      <c r="AN84" s="67">
+      <c r="AN84" s="56">
         <v>33</v>
       </c>
       <c r="AO84" s="44"/>
@@ -11311,10 +11311,10 @@
       <c r="AV84" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC84" s="67">
+      <c r="BC84" s="56">
         <v>48</v>
       </c>
-      <c r="BD84" s="67">
+      <c r="BD84" s="56">
         <v>48</v>
       </c>
       <c r="BE84" s="44"/>
@@ -11334,10 +11334,10 @@
         <v>5</v>
       </c>
       <c r="BQ84" s="36"/>
-      <c r="BS84" s="67">
+      <c r="BS84" s="56">
         <v>63</v>
       </c>
-      <c r="BT84" s="67">
+      <c r="BT84" s="56">
         <v>43</v>
       </c>
       <c r="BU84" s="44"/>
@@ -11360,7 +11360,7 @@
       <c r="CF84" s="18"/>
       <c r="CG84" s="6"/>
     </row>
-    <row r="85" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="5"/>
       <c r="B85" s="20"/>
       <c r="C85" s="5"/>
@@ -11377,10 +11377,10 @@
       <c r="A86" s="5"/>
       <c r="B86" s="20"/>
       <c r="C86" s="5"/>
-      <c r="G86" s="67">
+      <c r="G86" s="56">
         <v>4</v>
       </c>
-      <c r="H86" s="67"/>
+      <c r="H86" s="56"/>
       <c r="I86" s="44" t="s">
         <v>31</v>
       </c>
@@ -11419,10 +11419,10 @@
       <c r="AF86" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM86" s="67">
+      <c r="AM86" s="56">
         <v>34</v>
       </c>
-      <c r="AN86" s="67">
+      <c r="AN86" s="56">
         <v>34</v>
       </c>
       <c r="AO86" s="44"/>
@@ -11441,10 +11441,10 @@
       <c r="AV86" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC86" s="67">
+      <c r="BC86" s="56">
         <v>49</v>
       </c>
-      <c r="BD86" s="67">
+      <c r="BD86" s="56">
         <v>49</v>
       </c>
       <c r="BE86" s="44"/>
@@ -11464,10 +11464,10 @@
         <v>5</v>
       </c>
       <c r="BQ86" s="36"/>
-      <c r="BS86" s="67">
+      <c r="BS86" s="56">
         <v>64</v>
       </c>
-      <c r="BT86" s="67">
+      <c r="BT86" s="56">
         <v>44</v>
       </c>
       <c r="BU86" s="44"/>
@@ -11490,20 +11490,20 @@
       <c r="CF86" s="18"/>
       <c r="CG86" s="6"/>
     </row>
-    <row r="87" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="5"/>
       <c r="B87" s="20"/>
       <c r="C87" s="5"/>
-      <c r="G87" s="67"/>
-      <c r="H87" s="67"/>
+      <c r="G87" s="56"/>
+      <c r="H87" s="56"/>
       <c r="I87" s="44"/>
       <c r="Y87" s="44"/>
-      <c r="AM87" s="67"/>
-      <c r="AN87" s="67"/>
+      <c r="AM87" s="56"/>
+      <c r="AN87" s="56"/>
       <c r="AO87" s="44"/>
       <c r="BE87" s="44"/>
-      <c r="BS87" s="67"/>
-      <c r="BT87" s="67"/>
+      <c r="BS87" s="56"/>
+      <c r="BT87" s="56"/>
       <c r="BU87" s="44"/>
       <c r="CE87" s="6"/>
       <c r="CF87" s="18"/>
@@ -11513,10 +11513,10 @@
       <c r="A88" s="5"/>
       <c r="B88" s="20"/>
       <c r="C88" s="5"/>
-      <c r="G88" s="67">
+      <c r="G88" s="56">
         <v>5</v>
       </c>
-      <c r="H88" s="67"/>
+      <c r="H88" s="56"/>
       <c r="I88" s="44" t="s">
         <v>31</v>
       </c>
@@ -11555,10 +11555,10 @@
       <c r="AF88" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM88" s="67">
+      <c r="AM88" s="56">
         <v>35</v>
       </c>
-      <c r="AN88" s="67">
+      <c r="AN88" s="56">
         <v>35</v>
       </c>
       <c r="AO88" s="44"/>
@@ -11577,10 +11577,10 @@
       <c r="AV88" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC88" s="67">
+      <c r="BC88" s="56">
         <v>50</v>
       </c>
-      <c r="BD88" s="67">
+      <c r="BD88" s="56">
         <v>50</v>
       </c>
       <c r="BE88" s="44"/>
@@ -11641,10 +11641,10 @@
       <c r="A90" s="5"/>
       <c r="B90" s="20"/>
       <c r="C90" s="5"/>
-      <c r="G90" s="67">
+      <c r="G90" s="56">
         <v>6</v>
       </c>
-      <c r="H90" s="67"/>
+      <c r="H90" s="56"/>
       <c r="I90" s="44" t="s">
         <v>31</v>
       </c>
@@ -11663,10 +11663,10 @@
       <c r="P90" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="W90" s="67">
+      <c r="W90" s="56">
         <v>21</v>
       </c>
-      <c r="X90" s="67">
+      <c r="X90" s="56">
         <v>21</v>
       </c>
       <c r="Y90" s="44"/>
@@ -11685,10 +11685,10 @@
       <c r="AF90" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM90" s="67">
+      <c r="AM90" s="56">
         <v>36</v>
       </c>
-      <c r="AN90" s="67">
+      <c r="AN90" s="56">
         <v>36</v>
       </c>
       <c r="AO90" s="44"/>
@@ -11707,10 +11707,10 @@
       <c r="AV90" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC90" s="67">
+      <c r="BC90" s="56">
         <v>51</v>
       </c>
-      <c r="BD90" s="67">
+      <c r="BD90" s="56">
         <v>36</v>
       </c>
       <c r="BE90" s="44"/>
@@ -11754,7 +11754,7 @@
       <c r="CF90" s="18"/>
       <c r="CG90" s="6"/>
     </row>
-    <row r="91" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="5"/>
       <c r="B91" s="20"/>
       <c r="C91" s="5"/>
@@ -11766,10 +11766,10 @@
       <c r="A92" s="5"/>
       <c r="B92" s="20"/>
       <c r="C92" s="5"/>
-      <c r="G92" s="67">
+      <c r="G92" s="56">
         <v>7</v>
       </c>
-      <c r="H92" s="67"/>
+      <c r="H92" s="56"/>
       <c r="I92" s="44" t="s">
         <v>31</v>
       </c>
@@ -11788,10 +11788,10 @@
       <c r="P92" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="W92" s="67">
+      <c r="W92" s="56">
         <v>22</v>
       </c>
-      <c r="X92" s="67">
+      <c r="X92" s="56">
         <v>22</v>
       </c>
       <c r="Y92" s="44"/>
@@ -11810,10 +11810,10 @@
       <c r="AF92" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM92" s="67">
+      <c r="AM92" s="56">
         <v>37</v>
       </c>
-      <c r="AN92" s="67">
+      <c r="AN92" s="56">
         <v>37</v>
       </c>
       <c r="AO92" s="44"/>
@@ -11832,10 +11832,10 @@
       <c r="AV92" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC92" s="67">
+      <c r="BC92" s="56">
         <v>52</v>
       </c>
-      <c r="BD92" s="67">
+      <c r="BD92" s="56">
         <v>37</v>
       </c>
       <c r="BE92" s="44"/>
@@ -11879,7 +11879,7 @@
       <c r="CF92" s="18"/>
       <c r="CG92" s="6"/>
     </row>
-    <row r="93" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="5"/>
       <c r="B93" s="20"/>
       <c r="C93" s="5"/>
@@ -11891,10 +11891,10 @@
       <c r="A94" s="5"/>
       <c r="B94" s="20"/>
       <c r="C94" s="5"/>
-      <c r="G94" s="67">
+      <c r="G94" s="56">
         <v>8</v>
       </c>
-      <c r="H94" s="67"/>
+      <c r="H94" s="56"/>
       <c r="I94" s="44" t="s">
         <v>31</v>
       </c>
@@ -11913,10 +11913,10 @@
       <c r="P94" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="W94" s="67">
+      <c r="W94" s="56">
         <v>23</v>
       </c>
-      <c r="X94" s="67">
+      <c r="X94" s="56">
         <v>23</v>
       </c>
       <c r="Y94" s="44"/>
@@ -11935,10 +11935,10 @@
       <c r="AF94" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM94" s="67">
+      <c r="AM94" s="56">
         <v>38</v>
       </c>
-      <c r="AN94" s="67">
+      <c r="AN94" s="56">
         <v>38</v>
       </c>
       <c r="AO94" s="44"/>
@@ -11957,10 +11957,10 @@
       <c r="AV94" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC94" s="67">
+      <c r="BC94" s="56">
         <v>53</v>
       </c>
-      <c r="BD94" s="67">
+      <c r="BD94" s="56">
         <v>38</v>
       </c>
       <c r="BE94" s="44"/>
@@ -12004,7 +12004,7 @@
       <c r="CF94" s="18"/>
       <c r="CG94" s="6"/>
     </row>
-    <row r="95" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="5"/>
       <c r="B95" s="20"/>
       <c r="C95" s="5"/>
@@ -12016,10 +12016,10 @@
       <c r="A96" s="5"/>
       <c r="B96" s="20"/>
       <c r="C96" s="5"/>
-      <c r="G96" s="67">
+      <c r="G96" s="56">
         <v>9</v>
       </c>
-      <c r="H96" s="67"/>
+      <c r="H96" s="56"/>
       <c r="I96" s="44" t="s">
         <v>31</v>
       </c>
@@ -12038,10 +12038,10 @@
       <c r="P96" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="W96" s="67">
+      <c r="W96" s="56">
         <v>24</v>
       </c>
-      <c r="X96" s="67">
+      <c r="X96" s="56">
         <v>24</v>
       </c>
       <c r="Y96" s="44"/>
@@ -12060,10 +12060,10 @@
       <c r="AF96" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM96" s="67">
+      <c r="AM96" s="56">
         <v>39</v>
       </c>
-      <c r="AN96" s="67">
+      <c r="AN96" s="56">
         <v>39</v>
       </c>
       <c r="AO96" s="44"/>
@@ -12082,10 +12082,10 @@
       <c r="AV96" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC96" s="67">
+      <c r="BC96" s="56">
         <v>54</v>
       </c>
-      <c r="BD96" s="67">
+      <c r="BD96" s="56">
         <v>39</v>
       </c>
       <c r="BE96" s="44"/>
@@ -12129,12 +12129,12 @@
       <c r="CF96" s="18"/>
       <c r="CG96" s="6"/>
     </row>
-    <row r="97" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="5"/>
       <c r="B97" s="20"/>
       <c r="C97" s="5"/>
-      <c r="W97" s="67"/>
-      <c r="X97" s="67"/>
+      <c r="W97" s="56"/>
+      <c r="X97" s="56"/>
       <c r="CE97" s="6"/>
       <c r="CF97" s="18"/>
       <c r="CG97" s="6"/>
@@ -12143,10 +12143,10 @@
       <c r="A98" s="5"/>
       <c r="B98" s="20"/>
       <c r="C98" s="5"/>
-      <c r="G98" s="67">
+      <c r="G98" s="56">
         <v>10</v>
       </c>
-      <c r="H98" s="67"/>
+      <c r="H98" s="56"/>
       <c r="I98" s="44" t="s">
         <v>31</v>
       </c>
@@ -12165,10 +12165,10 @@
       <c r="P98" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="W98" s="67">
+      <c r="W98" s="56">
         <v>25</v>
       </c>
-      <c r="X98" s="67">
+      <c r="X98" s="56">
         <v>25</v>
       </c>
       <c r="Y98" s="44"/>
@@ -12187,10 +12187,10 @@
       <c r="AF98" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM98" s="67">
+      <c r="AM98" s="56">
         <v>40</v>
       </c>
-      <c r="AN98" s="67">
+      <c r="AN98" s="56">
         <v>40</v>
       </c>
       <c r="AO98" s="44"/>
@@ -12209,10 +12209,10 @@
       <c r="AV98" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC98" s="67">
+      <c r="BC98" s="56">
         <v>55</v>
       </c>
-      <c r="BD98" s="67">
+      <c r="BD98" s="56">
         <v>40</v>
       </c>
       <c r="BE98" s="44"/>
@@ -12273,10 +12273,10 @@
       <c r="A100" s="5"/>
       <c r="B100" s="20"/>
       <c r="C100" s="5"/>
-      <c r="G100" s="67">
+      <c r="G100" s="56">
         <v>11</v>
       </c>
-      <c r="H100" s="67">
+      <c r="H100" s="56">
         <v>11</v>
       </c>
       <c r="I100" s="44" t="s">
@@ -12317,10 +12317,10 @@
       <c r="AF100" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM100" s="67">
+      <c r="AM100" s="56">
         <v>41</v>
       </c>
-      <c r="AN100" s="67">
+      <c r="AN100" s="56">
         <v>36</v>
       </c>
       <c r="AO100" s="44"/>
@@ -12339,10 +12339,10 @@
       <c r="AV100" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC100" s="67">
+      <c r="BC100" s="56">
         <v>56</v>
       </c>
-      <c r="BD100" s="67">
+      <c r="BD100" s="56">
         <v>41</v>
       </c>
       <c r="BE100" s="44"/>
@@ -12386,7 +12386,7 @@
       <c r="CF100" s="18"/>
       <c r="CG100" s="6"/>
     </row>
-    <row r="101" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="5"/>
       <c r="B101" s="20"/>
       <c r="C101" s="5"/>
@@ -12398,10 +12398,10 @@
       <c r="A102" s="5"/>
       <c r="B102" s="20"/>
       <c r="C102" s="5"/>
-      <c r="G102" s="67">
+      <c r="G102" s="56">
         <v>12</v>
       </c>
-      <c r="H102" s="67">
+      <c r="H102" s="56">
         <v>12</v>
       </c>
       <c r="I102" s="44" t="s">
@@ -12442,10 +12442,10 @@
       <c r="AF102" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM102" s="67">
+      <c r="AM102" s="56">
         <v>42</v>
       </c>
-      <c r="AN102" s="67">
+      <c r="AN102" s="56">
         <v>37</v>
       </c>
       <c r="AO102" s="44"/>
@@ -12464,10 +12464,10 @@
       <c r="AV102" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC102" s="67">
+      <c r="BC102" s="56">
         <v>57</v>
       </c>
-      <c r="BD102" s="67">
+      <c r="BD102" s="56">
         <v>42</v>
       </c>
       <c r="BE102" s="44"/>
@@ -12511,7 +12511,7 @@
       <c r="CF102" s="18"/>
       <c r="CG102" s="6"/>
     </row>
-    <row r="103" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="5"/>
       <c r="B103" s="20"/>
       <c r="C103" s="5"/>
@@ -12523,10 +12523,10 @@
       <c r="A104" s="5"/>
       <c r="B104" s="20"/>
       <c r="C104" s="5"/>
-      <c r="G104" s="67">
+      <c r="G104" s="56">
         <v>13</v>
       </c>
-      <c r="H104" s="67">
+      <c r="H104" s="56">
         <v>13</v>
       </c>
       <c r="I104" s="44" t="s">
@@ -12567,10 +12567,10 @@
       <c r="AF104" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM104" s="67">
+      <c r="AM104" s="56">
         <v>43</v>
       </c>
-      <c r="AN104" s="67">
+      <c r="AN104" s="56">
         <v>38</v>
       </c>
       <c r="AO104" s="44"/>
@@ -12589,10 +12589,10 @@
       <c r="AV104" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC104" s="67">
+      <c r="BC104" s="56">
         <v>58</v>
       </c>
-      <c r="BD104" s="67">
+      <c r="BD104" s="56">
         <v>43</v>
       </c>
       <c r="BE104" s="44"/>
@@ -12636,7 +12636,7 @@
       <c r="CF104" s="18"/>
       <c r="CG104" s="6"/>
     </row>
-    <row r="105" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="5"/>
       <c r="B105" s="20"/>
       <c r="C105" s="5"/>
@@ -12648,10 +12648,10 @@
       <c r="A106" s="5"/>
       <c r="B106" s="20"/>
       <c r="C106" s="5"/>
-      <c r="G106" s="67">
+      <c r="G106" s="56">
         <v>14</v>
       </c>
-      <c r="H106" s="67">
+      <c r="H106" s="56">
         <v>14</v>
       </c>
       <c r="I106" s="44" t="s">
@@ -12692,10 +12692,10 @@
       <c r="AF106" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM106" s="67">
+      <c r="AM106" s="56">
         <v>44</v>
       </c>
-      <c r="AN106" s="67">
+      <c r="AN106" s="56">
         <v>39</v>
       </c>
       <c r="AO106" s="44"/>
@@ -12714,10 +12714,10 @@
       <c r="AV106" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC106" s="67">
+      <c r="BC106" s="56">
         <v>59</v>
       </c>
-      <c r="BD106" s="67">
+      <c r="BD106" s="56">
         <v>44</v>
       </c>
       <c r="BE106" s="44"/>
@@ -12761,14 +12761,14 @@
       <c r="CF106" s="18"/>
       <c r="CG106" s="6"/>
     </row>
-    <row r="107" spans="1:85" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:85" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="5"/>
       <c r="B107" s="20"/>
       <c r="C107" s="5"/>
-      <c r="G107" s="67"/>
-      <c r="H107" s="67"/>
-      <c r="BC107" s="67"/>
-      <c r="BD107" s="67"/>
+      <c r="G107" s="56"/>
+      <c r="H107" s="56"/>
+      <c r="BC107" s="56"/>
+      <c r="BD107" s="56"/>
       <c r="CE107" s="6"/>
       <c r="CF107" s="18"/>
       <c r="CG107" s="6"/>
@@ -12777,10 +12777,10 @@
       <c r="A108" s="5"/>
       <c r="B108" s="20"/>
       <c r="C108" s="5"/>
-      <c r="G108" s="67">
+      <c r="G108" s="56">
         <v>15</v>
       </c>
-      <c r="H108" s="67">
+      <c r="H108" s="56">
         <v>15</v>
       </c>
       <c r="I108" s="44" t="s">
@@ -12821,10 +12821,10 @@
       <c r="AF108" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AM108" s="67">
+      <c r="AM108" s="56">
         <v>45</v>
       </c>
-      <c r="AN108" s="67">
+      <c r="AN108" s="56">
         <v>40</v>
       </c>
       <c r="AO108" s="44"/>
@@ -12843,10 +12843,10 @@
       <c r="AV108" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="BC108" s="67">
+      <c r="BC108" s="56">
         <v>60</v>
       </c>
-      <c r="BD108" s="67">
+      <c r="BD108" s="56">
         <v>45</v>
       </c>
       <c r="BE108" s="44"/>
@@ -13156,25 +13156,60 @@
     <row r="115" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="93">
-    <mergeCell ref="W97:X97"/>
-    <mergeCell ref="AM80:AN80"/>
-    <mergeCell ref="AM82:AN82"/>
-    <mergeCell ref="AM84:AN84"/>
-    <mergeCell ref="AM86:AN86"/>
-    <mergeCell ref="AM87:AN87"/>
-    <mergeCell ref="AM90:AN90"/>
-    <mergeCell ref="G94:H94"/>
-    <mergeCell ref="W94:X94"/>
-    <mergeCell ref="AT54:CD54"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="BC80:BD80"/>
-    <mergeCell ref="BS80:BT80"/>
-    <mergeCell ref="G82:H82"/>
-    <mergeCell ref="BC82:BD82"/>
-    <mergeCell ref="BS82:BT82"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="BC84:BD84"/>
-    <mergeCell ref="BS84:BT84"/>
+    <mergeCell ref="D9:AP9"/>
+    <mergeCell ref="D4:AP4"/>
+    <mergeCell ref="D5:AP5"/>
+    <mergeCell ref="D6:AP6"/>
+    <mergeCell ref="D7:AP7"/>
+    <mergeCell ref="D8:AP8"/>
+    <mergeCell ref="AU64:AV64"/>
+    <mergeCell ref="AU66:AV66"/>
+    <mergeCell ref="AU68:AV68"/>
+    <mergeCell ref="AU70:AV70"/>
+    <mergeCell ref="D10:AP10"/>
+    <mergeCell ref="D19:AP20"/>
+    <mergeCell ref="AT46:CD46"/>
+    <mergeCell ref="AT19:BM20"/>
+    <mergeCell ref="BZ19:CD20"/>
+    <mergeCell ref="BP19:BV20"/>
+    <mergeCell ref="BS68:BT68"/>
+    <mergeCell ref="BS70:BT70"/>
+    <mergeCell ref="BS72:BT72"/>
+    <mergeCell ref="BG68:BH68"/>
+    <mergeCell ref="BG70:BH70"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="W98:X98"/>
+    <mergeCell ref="AM98:AN98"/>
+    <mergeCell ref="BC98:BD98"/>
+    <mergeCell ref="AU71:AV71"/>
+    <mergeCell ref="AU72:AV72"/>
+    <mergeCell ref="D78:CD78"/>
+    <mergeCell ref="AM94:AN94"/>
+    <mergeCell ref="BC94:BD94"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="W96:X96"/>
+    <mergeCell ref="AM96:AN96"/>
+    <mergeCell ref="BC96:BD96"/>
+    <mergeCell ref="BG72:BH72"/>
+    <mergeCell ref="G90:H90"/>
+    <mergeCell ref="W90:X90"/>
+    <mergeCell ref="G108:H108"/>
+    <mergeCell ref="AM108:AN108"/>
+    <mergeCell ref="BC108:BD108"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="BC107:BD107"/>
+    <mergeCell ref="G100:H100"/>
+    <mergeCell ref="AM100:AN100"/>
+    <mergeCell ref="BC100:BD100"/>
+    <mergeCell ref="AM106:AN106"/>
+    <mergeCell ref="BC106:BD106"/>
+    <mergeCell ref="G104:H104"/>
+    <mergeCell ref="AM104:AN104"/>
+    <mergeCell ref="BC104:BD104"/>
+    <mergeCell ref="G106:H106"/>
+    <mergeCell ref="G102:H102"/>
+    <mergeCell ref="AM102:AN102"/>
+    <mergeCell ref="BC102:BD102"/>
     <mergeCell ref="AT48:CD52"/>
     <mergeCell ref="BC90:BD90"/>
     <mergeCell ref="G92:H92"/>
@@ -13191,64 +13226,29 @@
     <mergeCell ref="AM88:AN88"/>
     <mergeCell ref="BG64:BH64"/>
     <mergeCell ref="BG66:BH66"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="AM100:AN100"/>
-    <mergeCell ref="BC100:BD100"/>
-    <mergeCell ref="AM106:AN106"/>
-    <mergeCell ref="BC106:BD106"/>
-    <mergeCell ref="G104:H104"/>
-    <mergeCell ref="AM104:AN104"/>
-    <mergeCell ref="BC104:BD104"/>
-    <mergeCell ref="G106:H106"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="AM102:AN102"/>
-    <mergeCell ref="BC102:BD102"/>
-    <mergeCell ref="G108:H108"/>
-    <mergeCell ref="AM108:AN108"/>
-    <mergeCell ref="BC108:BD108"/>
-    <mergeCell ref="G107:H107"/>
-    <mergeCell ref="BC107:BD107"/>
-    <mergeCell ref="G98:H98"/>
-    <mergeCell ref="W98:X98"/>
-    <mergeCell ref="AM98:AN98"/>
-    <mergeCell ref="BC98:BD98"/>
-    <mergeCell ref="AU71:AV71"/>
-    <mergeCell ref="AU72:AV72"/>
-    <mergeCell ref="D78:CD78"/>
-    <mergeCell ref="AM94:AN94"/>
-    <mergeCell ref="BC94:BD94"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="W96:X96"/>
-    <mergeCell ref="AM96:AN96"/>
-    <mergeCell ref="BC96:BD96"/>
-    <mergeCell ref="BG72:BH72"/>
-    <mergeCell ref="G90:H90"/>
-    <mergeCell ref="W90:X90"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="W94:X94"/>
+    <mergeCell ref="AT54:CD54"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="BC80:BD80"/>
+    <mergeCell ref="BS80:BT80"/>
+    <mergeCell ref="G82:H82"/>
+    <mergeCell ref="BC82:BD82"/>
+    <mergeCell ref="BS82:BT82"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="BC84:BD84"/>
+    <mergeCell ref="BS84:BT84"/>
     <mergeCell ref="BS64:BT64"/>
     <mergeCell ref="BS66:BT66"/>
     <mergeCell ref="AT62:CD62"/>
     <mergeCell ref="D77:CD77"/>
-    <mergeCell ref="BS68:BT68"/>
-    <mergeCell ref="BS70:BT70"/>
-    <mergeCell ref="BS72:BT72"/>
-    <mergeCell ref="BG68:BH68"/>
-    <mergeCell ref="BG70:BH70"/>
-    <mergeCell ref="AU64:AV64"/>
-    <mergeCell ref="AU66:AV66"/>
-    <mergeCell ref="AU68:AV68"/>
-    <mergeCell ref="AU70:AV70"/>
-    <mergeCell ref="D10:AP10"/>
-    <mergeCell ref="D19:AP20"/>
-    <mergeCell ref="AT46:CD46"/>
-    <mergeCell ref="D9:AP9"/>
-    <mergeCell ref="D4:AP4"/>
-    <mergeCell ref="D5:AP5"/>
-    <mergeCell ref="D6:AP6"/>
-    <mergeCell ref="D7:AP7"/>
-    <mergeCell ref="D8:AP8"/>
-    <mergeCell ref="AT19:BM20"/>
-    <mergeCell ref="BZ19:CD20"/>
-    <mergeCell ref="BP19:BV20"/>
+    <mergeCell ref="W97:X97"/>
+    <mergeCell ref="AM80:AN80"/>
+    <mergeCell ref="AM82:AN82"/>
+    <mergeCell ref="AM84:AN84"/>
+    <mergeCell ref="AM86:AN86"/>
+    <mergeCell ref="AM87:AN87"/>
+    <mergeCell ref="AM90:AN90"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="73" orientation="portrait" verticalDpi="0"/>

</xml_diff>